<commit_message>
update simulation reports and add conversion script
</commit_message>
<xml_diff>
--- a/selenium_tests/reports/selenium_report.xlsx
+++ b/selenium_tests/reports/selenium_report.xlsx
@@ -11,12 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="826" uniqueCount="527">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="826" uniqueCount="533">
   <si>
     <t>VolunteerSync Flutter Web — Selenium E2E Test Report</t>
   </si>
   <si>
-    <t xml:space="preserve">  Browser: Chrome  |  Target: Flutter Web (localhost:8080)  |  Generated: 13/6/2026, 10:00:29 am</t>
+    <t xml:space="preserve">  Browser: Chrome  |  Target: Flutter Web (localhost:8080)  |  Generated: 14/6/2026, 5:10:45 pm</t>
   </si>
   <si>
     <t xml:space="preserve">  EXECUTION SUMMARY</t>
@@ -40,13 +40,13 @@
     <t>Total Duration</t>
   </si>
   <si>
-    <t>102.28s</t>
+    <t>103.59s</t>
   </si>
   <si>
     <t>Run At</t>
   </si>
   <si>
-    <t>13/6/2026, 10:00:29 am</t>
+    <t>14/6/2026, 5:10:45 pm</t>
   </si>
   <si>
     <t>Test ID</t>
@@ -91,10 +91,10 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:25.670Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:26.822Z</t>
+    <t>2026-06-14T11:40:41.617Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:43.278Z</t>
   </si>
   <si>
     <t>No errors. Flow completed successfully.</t>
@@ -109,10 +109,10 @@
     <t>Verify hero section headline text is present and visible on page load.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:25.712Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:26.992Z</t>
+    <t>2026-06-14T11:40:41.660Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:43.390Z</t>
   </si>
   <si>
     <t>TC-003</t>
@@ -124,10 +124,10 @@
     <t>Verify the subtitle/description paragraph appears below the hero title.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:25.745Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:27.200Z</t>
+    <t>2026-06-14T11:40:41.699Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:42.434Z</t>
   </si>
   <si>
     <t>TC-004</t>
@@ -139,10 +139,10 @@
     <t>Verify the gradient VolunteerSync logo/icon is visible in the header.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:25.784Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:26.517Z</t>
+    <t>2026-06-14T11:40:41.741Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:43.381Z</t>
   </si>
   <si>
     <t>TC-005</t>
@@ -154,10 +154,10 @@
     <t>Verify "Get Started" primary CTA button renders and is clickable.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:25.825Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:27.393Z</t>
+    <t>2026-06-14T11:40:41.777Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:42.215Z</t>
   </si>
   <si>
     <t>TC-006</t>
@@ -169,10 +169,10 @@
     <t>Verify clicking "Sign In" navigates the browser to /login route.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:25.866Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:26.366Z</t>
+    <t>2026-06-14T11:40:41.818Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:42.474Z</t>
   </si>
   <si>
     <t>TC-007</t>
@@ -184,10 +184,10 @@
     <t>Verify the features/benefits section is displayed below the hero.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:25.902Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:27.416Z</t>
+    <t>2026-06-14T11:40:41.850Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:43.089Z</t>
   </si>
   <si>
     <t>TC-008</t>
@@ -199,10 +199,10 @@
     <t>Verify numerical statistics blocks (e.g. "1,000+ Volunteers") appear.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:25.947Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:26.973Z</t>
+    <t>2026-06-14T11:40:41.882Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:42.638Z</t>
   </si>
   <si>
     <t>TC-009</t>
@@ -214,10 +214,10 @@
     <t>Verify the browser &lt;title&gt; tag contains "VolunteerSync".</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:25.988Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:26.892Z</t>
+    <t>2026-06-14T11:40:41.922Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:42.682Z</t>
   </si>
   <si>
     <t>TC-010</t>
@@ -229,10 +229,10 @@
     <t>Verify page does not overflow on 1280x900 viewport resolution.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:26.025Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:26.500Z</t>
+    <t>2026-06-14T11:40:41.959Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:43.384Z</t>
   </si>
   <si>
     <t>TC-011</t>
@@ -247,10 +247,10 @@
     <t>Verify /login route loads the login screen without errors.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:26.061Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:27.640Z</t>
+    <t>2026-06-14T11:40:41.998Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:42.997Z</t>
   </si>
   <si>
     <t>TC-012</t>
@@ -262,10 +262,10 @@
     <t>Verify the email input field is rendered and accepts keyboard input.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:26.093Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:26.503Z</t>
+    <t>2026-06-14T11:40:42.040Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:43.370Z</t>
   </si>
   <si>
     <t>TC-013</t>
@@ -277,10 +277,10 @@
     <t>Verify the password field is rendered and masks characters by default.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:26.125Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:27.129Z</t>
+    <t>2026-06-14T11:40:42.074Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:43.324Z</t>
   </si>
   <si>
     <t>TC-014</t>
@@ -292,10 +292,10 @@
     <t>Verify the eye icon toggles the password field to plaintext and back.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:26.165Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:27.368Z</t>
+    <t>2026-06-14T11:40:42.116Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:42.739Z</t>
   </si>
   <si>
     <t>TC-015</t>
@@ -307,10 +307,10 @@
     <t>Verify submitting with no email shows "Enter a valid email" error text.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:26.196Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:27.023Z</t>
+    <t>2026-06-14T11:40:42.158Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:42.825Z</t>
   </si>
   <si>
     <t>TC-016</t>
@@ -322,10 +322,10 @@
     <t>Verify entering "invalidemail" (no @) shows field validation warning.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:26.235Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:26.864Z</t>
+    <t>2026-06-14T11:40:42.201Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:42.567Z</t>
   </si>
   <si>
     <t>TC-017</t>
@@ -337,10 +337,10 @@
     <t>Verify entering a password under 6 characters shows "Min 6 characters".</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:26.276Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:27.559Z</t>
+    <t>2026-06-14T11:40:42.241Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:43.789Z</t>
   </si>
   <si>
     <t>TC-018</t>
@@ -352,10 +352,10 @@
     <t>Verify "Forgot password?" link opens /forgot-password route.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:26.307Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:27.438Z</t>
+    <t>2026-06-14T11:40:42.283Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:43.701Z</t>
   </si>
   <si>
     <t>TC-019</t>
@@ -367,10 +367,10 @@
     <t>Verify "Sign up free →" navigates to /register route.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:26.339Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:27.413Z</t>
+    <t>2026-06-14T11:40:42.313Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:43.301Z</t>
   </si>
   <si>
     <t>TC-020</t>
@@ -382,10 +382,10 @@
     <t>Verify back arrow button returns to the / landing screen.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:26.381Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:27.939Z</t>
+    <t>2026-06-14T11:40:42.350Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:43.872Z</t>
   </si>
   <si>
     <t>TC-021</t>
@@ -397,10 +397,10 @@
     <t>Verify Sign In button transitions to a loading spinner on submit.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:26.418Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:27.635Z</t>
+    <t>2026-06-14T11:40:42.383Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:43.594Z</t>
   </si>
   <si>
     <t>TC-022</t>
@@ -412,10 +412,10 @@
     <t>Verify incorrect credentials show an error banner on the login form.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:26.458Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:28.063Z</t>
+    <t>2026-06-14T11:40:42.417Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:43.452Z</t>
   </si>
   <si>
     <t>TC-023</t>
@@ -427,10 +427,10 @@
     <t>Enter alex@volunteersync.io / password123 and confirm /dashboard redirect.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:26.490Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:26.984Z</t>
+    <t>2026-06-14T11:40:42.452Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:43.611Z</t>
   </si>
   <si>
     <t>TC-024</t>
@@ -442,10 +442,10 @@
     <t>Verify direct navigation to /dashboard redirects to /login if not logged in.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:26.530Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:28.044Z</t>
+    <t>2026-06-14T11:40:42.490Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:43.315Z</t>
   </si>
   <si>
     <t>TC-025</t>
@@ -460,10 +460,10 @@
     <t>Verify /register route renders the onboarding form correctly.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:26.570Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:27.981Z</t>
+    <t>2026-06-14T11:40:42.520Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:43.738Z</t>
   </si>
   <si>
     <t>TC-026</t>
@@ -475,10 +475,10 @@
     <t>Verify Name, Email, Password, and Role fields are present.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:26.603Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:27.169Z</t>
+    <t>2026-06-14T11:40:42.560Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:44.265Z</t>
   </si>
   <si>
     <t>TC-027</t>
@@ -490,10 +490,10 @@
     <t>Verify submitting a blank register form shows required field errors.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:26.635Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:28.303Z</t>
+    <t>2026-06-14T11:40:42.599Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:44.160Z</t>
   </si>
   <si>
     <t>TC-028</t>
@@ -505,10 +505,10 @@
     <t>Verify "Sign in →" link navigates back to /login page.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:26.668Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:27.513Z</t>
+    <t>2026-06-14T11:40:42.640Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:43.167Z</t>
   </si>
   <si>
     <t>TC-029</t>
@@ -523,7 +523,10 @@
     <t>Verify /forgot-password page loads the reset form.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:26.708Z</t>
+    <t>2026-06-14T11:40:42.681Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:44.383Z</t>
   </si>
   <si>
     <t>TC-030</t>
@@ -535,10 +538,10 @@
     <t>Enter email and verify success state screen displays after submit.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:26.740Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:27.256Z</t>
+    <t>2026-06-14T11:40:42.725Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:43.999Z</t>
   </si>
   <si>
     <t>TC-031</t>
@@ -553,7 +556,10 @@
     <t>Verify /dashboard route renders after successful authentication.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:26.774Z</t>
+    <t>2026-06-14T11:40:42.758Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:43.269Z</t>
   </si>
   <si>
     <t>TC-032</t>
@@ -565,10 +571,10 @@
     <t>Verify the left sidebar is displayed with all navigation menu items.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:26.816Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:28.451Z</t>
+    <t>2026-06-14T11:40:42.790Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:44.193Z</t>
   </si>
   <si>
     <t>TC-033</t>
@@ -580,10 +586,7 @@
     <t>Verify the "Total Volunteers" statistic card is present with a number.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:26.848Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:28.468Z</t>
+    <t>2026-06-14T11:40:44.229Z</t>
   </si>
   <si>
     <t>TC-034</t>
@@ -595,10 +598,10 @@
     <t>Verify the "Active Events" KPI card displays correct metric data.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:26.888Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:27.353Z</t>
+    <t>2026-06-14T11:40:42.866Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:43.297Z</t>
   </si>
   <si>
     <t>TC-035</t>
@@ -610,10 +613,10 @@
     <t>Verify the "Total Hours" KPI metric card renders with a number value.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:26.929Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:27.902Z</t>
+    <t>2026-06-14T11:40:42.902Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:44.620Z</t>
   </si>
   <si>
     <t>TC-036</t>
@@ -625,10 +628,10 @@
     <t>Verify the "Retention Rate" percentage card is displayed on dashboard.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:26.969Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:28.686Z</t>
+    <t>2026-06-14T11:40:42.936Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:43.672Z</t>
   </si>
   <si>
     <t>TC-037</t>
@@ -640,10 +643,10 @@
     <t>Verify the line chart rendering the volunteer growth trend is present.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:27.004Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:27.924Z</t>
+    <t>2026-06-14T11:40:42.980Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:43.373Z</t>
   </si>
   <si>
     <t>TC-038</t>
@@ -655,10 +658,10 @@
     <t>Verify the attendance bar chart is rendered with visible columns.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:27.036Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:28.504Z</t>
+    <t>2026-06-14T11:40:43.019Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:43.426Z</t>
   </si>
   <si>
     <t>TC-039</t>
@@ -670,10 +673,10 @@
     <t>Verify the category distribution pie chart is visible on dashboard.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:27.077Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:27.909Z</t>
+    <t>2026-06-14T11:40:43.061Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:43.763Z</t>
   </si>
   <si>
     <t>TC-040</t>
@@ -685,10 +688,10 @@
     <t>Verify the activity feed list shows timestamped volunteer actions.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:27.109Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:28.749Z</t>
+    <t>2026-06-14T11:40:43.100Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:44.211Z</t>
   </si>
   <si>
     <t>TC-041</t>
@@ -700,10 +703,10 @@
     <t>Verify the Volt AI insight recommendation widget is visible.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:27.149Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:27.566Z</t>
+    <t>2026-06-14T11:40:43.132Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:44.558Z</t>
   </si>
   <si>
     <t>TC-042</t>
@@ -715,10 +718,10 @@
     <t>Verify clicking the collapse arrow narrows the sidebar to icon-only mode.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:27.181Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:28.622Z</t>
+    <t>2026-06-14T11:40:43.168Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:44.753Z</t>
   </si>
   <si>
     <t>TC-043</t>
@@ -730,10 +733,10 @@
     <t>Verify clicking the expand icon re-opens the sidebar to full width.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:27.217Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:28.232Z</t>
+    <t>2026-06-14T11:40:43.199Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:43.697Z</t>
   </si>
   <si>
     <t>TC-044</t>
@@ -745,10 +748,10 @@
     <t>Verify the "Dashboard" nav item is highlighted/active on /dashboard.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:27.248Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:28.357Z</t>
+    <t>2026-06-14T11:40:43.241Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:43.622Z</t>
   </si>
   <si>
     <t>TC-045</t>
@@ -760,10 +763,10 @@
     <t>Verify the logged-in user name appears in the sidebar bottom section.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:27.290Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:27.759Z</t>
+    <t>2026-06-14T11:40:43.285Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:44.028Z</t>
   </si>
   <si>
     <t>TC-046</t>
@@ -778,10 +781,10 @@
     <t>Click "Volunteers" in sidebar and verify /volunteers route loads.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:27.329Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:28.584Z</t>
+    <t>2026-06-14T11:40:43.331Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:44.452Z</t>
   </si>
   <si>
     <t>TC-047</t>
@@ -793,10 +796,10 @@
     <t>Verify the volunteer listing grid/list is populated with cards.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:27.372Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:27.901Z</t>
+    <t>2026-06-14T11:40:43.366Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:44.026Z</t>
   </si>
   <si>
     <t>TC-048</t>
@@ -808,7 +811,10 @@
     <t>Verify the search input field is visible and accepts text.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:28.932Z</t>
+    <t>2026-06-14T11:40:43.408Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:44.889Z</t>
   </si>
   <si>
     <t>TC-049</t>
@@ -820,10 +826,10 @@
     <t>Type "Alex" in search and verify filtered results appear.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:27.445Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:28.281Z</t>
+    <t>2026-06-14T11:40:43.444Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:44.511Z</t>
   </si>
   <si>
     <t>TC-050</t>
@@ -835,10 +841,10 @@
     <t>Type "zzznoresult" in search and verify empty state message shows.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:27.484Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:28.854Z</t>
+    <t>2026-06-14T11:40:43.490Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:44.734Z</t>
   </si>
   <si>
     <t>TC-051</t>
@@ -850,10 +856,10 @@
     <t>Click "All" filter chip and verify full volunteer list renders.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:27.524Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:28.474Z</t>
+    <t>2026-06-14T11:40:43.532Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:44.384Z</t>
   </si>
   <si>
     <t>TC-052</t>
@@ -865,7 +871,10 @@
     <t>Click "Active" chip and verify only active volunteers appear.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:28.953Z</t>
+    <t>2026-06-14T11:40:43.575Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:44.053Z</t>
   </si>
   <si>
     <t>TC-053</t>
@@ -877,10 +886,10 @@
     <t>Click "Inactive" chip and verify filtered-down inactive members.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:27.598Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:28.221Z</t>
+    <t>2026-06-14T11:40:43.616Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:44.514Z</t>
   </si>
   <si>
     <t>TC-054</t>
@@ -892,10 +901,10 @@
     <t>Click "Pending" chip and verify pending members list.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:27.637Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:28.788Z</t>
+    <t>2026-06-14T11:40:43.653Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:44.487Z</t>
   </si>
   <si>
     <t>TC-055</t>
@@ -907,10 +916,10 @@
     <t>Verify each volunteer list card shows an avatar with name initials.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:27.679Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:28.305Z</t>
+    <t>2026-06-14T11:40:43.696Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:45.289Z</t>
   </si>
   <si>
     <t>TC-056</t>
@@ -922,10 +931,10 @@
     <t>Click a volunteer card and verify the profile detail sheet slides in.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:27.717Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:28.135Z</t>
+    <t>2026-06-14T11:40:43.730Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:45.409Z</t>
   </si>
   <si>
     <t>TC-057</t>
@@ -937,10 +946,10 @@
     <t>Verify the volunteer email is visible in the opened profile sheet.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:27.755Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:29.063Z</t>
+    <t>2026-06-14T11:40:43.764Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:44.141Z</t>
   </si>
   <si>
     <t>TC-058</t>
@@ -952,7 +961,10 @@
     <t>Verify cumulative hours are listed in the volunteer detail view.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:27.787Z</t>
+    <t>2026-06-14T11:40:43.805Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:44.920Z</t>
   </si>
   <si>
     <t>TC-059</t>
@@ -964,10 +976,10 @@
     <t>Verify team/group badge labels appear in the profile detail sheet.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:27.826Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:28.184Z</t>
+    <t>2026-06-14T11:40:43.840Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:44.828Z</t>
   </si>
   <si>
     <t>TC-060</t>
@@ -979,10 +991,10 @@
     <t>Click outside or close button and verify the profile sheet dismisses.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:27.866Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:28.597Z</t>
+    <t>2026-06-14T11:40:43.884Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:45.383Z</t>
   </si>
   <si>
     <t>TC-061</t>
@@ -997,10 +1009,10 @@
     <t>Click "Events" sidebar item and verify /events route loads.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:27.897Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:28.577Z</t>
+    <t>2026-06-14T11:40:43.915Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:45.506Z</t>
   </si>
   <si>
     <t>TC-062</t>
@@ -1012,10 +1024,10 @@
     <t>Verify at least one event card is displayed in the events list.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:27.938Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:29.437Z</t>
+    <t>2026-06-14T11:40:43.949Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:45.469Z</t>
   </si>
   <si>
     <t>TC-063</t>
@@ -1027,10 +1039,10 @@
     <t>Verify event card titles (e.g. "Food Drive") are visible.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:27.978Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:29.344Z</t>
+    <t>2026-06-14T11:40:43.979Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:44.614Z</t>
   </si>
   <si>
     <t>TC-064</t>
@@ -1042,10 +1054,10 @@
     <t>Verify event date labels are formatted and displayed per card.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:28.017Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:29.587Z</t>
+    <t>2026-06-14T11:40:44.019Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:44.984Z</t>
   </si>
   <si>
     <t>TC-065</t>
@@ -1057,10 +1069,10 @@
     <t>Verify location text is shown on each event card.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:28.059Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:28.410Z</t>
+    <t>2026-06-14T11:40:44.061Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:45.729Z</t>
   </si>
   <si>
     <t>TC-066</t>
@@ -1072,10 +1084,10 @@
     <t>Verify volunteer capacity progress bar renders on event cards.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:28.091Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:29.129Z</t>
+    <t>2026-06-14T11:40:44.102Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:45.658Z</t>
   </si>
   <si>
     <t>TC-067</t>
@@ -1087,10 +1099,10 @@
     <t>Verify category classification badge is shown per event.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:28.124Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:29.070Z</t>
+    <t>2026-06-14T11:40:44.144Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:45.614Z</t>
   </si>
   <si>
     <t>TC-068</t>
@@ -1102,10 +1114,10 @@
     <t>Type "Food" in events search and verify matching cards appear.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:28.163Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:29.865Z</t>
+    <t>2026-06-14T11:40:44.180Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:44.656Z</t>
   </si>
   <si>
     <t>TC-069</t>
@@ -1117,10 +1129,10 @@
     <t>Click an event card and verify the event detail sheet expands.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:28.195Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:29.392Z</t>
+    <t>2026-06-14T11:40:44.226Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:44.968Z</t>
   </si>
   <si>
     <t>TC-070</t>
@@ -1132,10 +1144,10 @@
     <t>Verify the event agenda/description paragraph is visible in sheet.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:28.235Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:28.853Z</t>
+    <t>2026-06-14T11:40:44.258Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:44.747Z</t>
   </si>
   <si>
     <t>TC-071</t>
@@ -1147,10 +1159,10 @@
     <t>Verify the list of assigned volunteers appears in event detail.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:28.276Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:29.501Z</t>
+    <t>2026-06-14T11:40:44.300Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:44.652Z</t>
   </si>
   <si>
     <t>TC-072</t>
@@ -1162,10 +1174,10 @@
     <t>Verify clicking close dismisses the event detail sheet.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:28.315Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:29.166Z</t>
+    <t>2026-06-14T11:40:44.341Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:45.696Z</t>
   </si>
   <si>
     <t>TC-073</t>
@@ -1180,10 +1192,10 @@
     <t>Click "Attendance" sidebar item and verify /attendance route loads.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:28.347Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:29.646Z</t>
+    <t>2026-06-14T11:40:44.385Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:44.886Z</t>
   </si>
   <si>
     <t>TC-074</t>
@@ -1195,10 +1207,10 @@
     <t>Verify checked-in count statistics are shown in a metrics bar.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:28.387Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:28.963Z</t>
+    <t>2026-06-14T11:40:44.423Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:45.597Z</t>
   </si>
   <si>
     <t>TC-075</t>
@@ -1210,10 +1222,10 @@
     <t>Verify the attendance log table is rendered with row records.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:28.419Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:29.424Z</t>
+    <t>2026-06-14T11:40:44.459Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:45.281Z</t>
   </si>
   <si>
     <t>TC-076</t>
@@ -1225,10 +1237,10 @@
     <t>Verify table columns (Volunteer, Event, Date, Duration) are labeled.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:28.457Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:28.856Z</t>
+    <t>2026-06-14T11:40:44.494Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:45.090Z</t>
   </si>
   <si>
     <t>TC-077</t>
@@ -1240,10 +1252,10 @@
     <t>Type a volunteer name in search and verify matching log rows.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:28.488Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:30.087Z</t>
+    <t>2026-06-14T11:40:44.525Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:45.510Z</t>
   </si>
   <si>
     <t>TC-078</t>
@@ -1255,10 +1267,10 @@
     <t>Filter attendance records by selecting a specific event.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:28.527Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:29.579Z</t>
+    <t>2026-06-14T11:40:44.568Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:44.965Z</t>
   </si>
   <si>
     <t>TC-079</t>
@@ -1270,10 +1282,10 @@
     <t>Verify the "Check-In" action button is present and clickable.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:28.562Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:30.032Z</t>
+    <t>2026-06-14T11:40:44.603Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:45.072Z</t>
   </si>
   <si>
     <t>TC-080</t>
@@ -1285,10 +1297,10 @@
     <t>Click Check-In and verify the volunteer selection dialog opens.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:28.592Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:29.906Z</t>
+    <t>2026-06-14T11:40:44.634Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:45.047Z</t>
   </si>
   <si>
     <t>TC-081</t>
@@ -1300,10 +1312,10 @@
     <t>Select event and volunteer in dialog, submit and verify toast confirmation.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:28.632Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:30.235Z</t>
+    <t>2026-06-14T11:40:44.667Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:46.268Z</t>
   </si>
   <si>
     <t>TC-082</t>
@@ -1315,10 +1327,10 @@
     <t>Click Export and verify download is triggered for the data.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:28.672Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:29.841Z</t>
+    <t>2026-06-14T11:40:44.709Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:45.656Z</t>
   </si>
   <si>
     <t>TC-083</t>
@@ -1333,10 +1345,10 @@
     <t>Click "Reports" sidebar item and verify /reports route loads.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:28.711Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:29.715Z</t>
+    <t>2026-06-14T11:40:44.744Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:45.309Z</t>
   </si>
   <si>
     <t>TC-084</t>
@@ -1348,7 +1360,10 @@
     <t>Verify multiple charts and analytics sections render on reports page.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:30.193Z</t>
+    <t>2026-06-14T11:40:44.776Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:46.220Z</t>
   </si>
   <si>
     <t>TC-085</t>
@@ -1360,10 +1375,10 @@
     <t>Verify a sortable top contributors table is present on reports screen.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:28.795Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:29.263Z</t>
+    <t>2026-06-14T11:40:44.822Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:45.646Z</t>
   </si>
   <si>
     <t>TC-086</t>
@@ -1375,10 +1390,10 @@
     <t>Verify a date filter/range picker is available on the reports screen.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:28.835Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:29.199Z</t>
+    <t>2026-06-14T11:40:44.855Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:45.211Z</t>
   </si>
   <si>
     <t>TC-087</t>
@@ -1393,10 +1408,10 @@
     <t>Click "AI Assistant" sidebar item and verify /ai-chat route loads.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:28.875Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:29.877Z</t>
+    <t>2026-06-14T11:40:44.901Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:46.449Z</t>
   </si>
   <si>
     <t>TC-088</t>
@@ -1408,10 +1423,10 @@
     <t>Verify "Volt" AI assistant header and intro message is displayed.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:28.915Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:29.515Z</t>
+    <t>2026-06-14T11:40:44.942Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:45.810Z</t>
   </si>
   <si>
     <t>TC-089</t>
@@ -1423,10 +1438,10 @@
     <t>Verify quick-prompt suggestion cards are rendered in the chat view.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:28.949Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:29.952Z</t>
+    <t>2026-06-14T11:40:44.985Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:45.464Z</t>
   </si>
   <si>
     <t>TC-090</t>
@@ -1438,10 +1453,10 @@
     <t>Verify the message input field is visible and accepts typed text.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:28.981Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:29.563Z</t>
+    <t>2026-06-14T11:40:45.026Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:46.202Z</t>
   </si>
   <si>
     <t>TC-091</t>
@@ -1453,10 +1468,10 @@
     <t>Type "Show upcoming events" and press Enter; verify message bubble appears.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:29.021Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:29.691Z</t>
+    <t>2026-06-14T11:40:45.069Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:46.101Z</t>
   </si>
   <si>
     <t>TC-092</t>
@@ -1468,10 +1483,10 @@
     <t>Verify Volt AI returns a response bubble with structured text.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:29.061Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:29.701Z</t>
+    <t>2026-06-14T11:40:45.109Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:45.857Z</t>
   </si>
   <si>
     <t>TC-093</t>
@@ -1483,7 +1498,10 @@
     <t>Type "Generate attendance report" and verify AI processes the request.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:29.093Z</t>
+    <t>2026-06-14T11:40:45.151Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:46.739Z</t>
   </si>
   <si>
     <t>TC-094</t>
@@ -1495,10 +1513,10 @@
     <t>Verify a typing animation/indicator appears while Volt computes reply.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:29.125Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:29.949Z</t>
+    <t>2026-06-14T11:40:45.195Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:46.552Z</t>
   </si>
   <si>
     <t>TC-095</t>
@@ -1513,10 +1531,10 @@
     <t>Click "Settings" sidebar item and verify /settings route loads.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:29.165Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:30.816Z</t>
+    <t>2026-06-14T11:40:45.234Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:45.606Z</t>
   </si>
   <si>
     <t>TC-096</t>
@@ -1528,10 +1546,10 @@
     <t>Verify user name, email, and role appear in the profile section.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:29.197Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:29.549Z</t>
+    <t>2026-06-14T11:40:45.271Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:46.767Z</t>
   </si>
   <si>
     <t>TC-097</t>
@@ -1543,10 +1561,10 @@
     <t>Verify Email/Push notification toggle switches are rendered.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:29.229Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:30.375Z</t>
+    <t>2026-06-14T11:40:45.306Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:46.597Z</t>
   </si>
   <si>
     <t>TC-098</t>
@@ -1558,10 +1576,10 @@
     <t>Click email notification switch and verify it changes state.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:29.269Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:30.471Z</t>
+    <t>2026-06-14T11:40:45.340Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:46.998Z</t>
   </si>
   <si>
     <t>TC-099</t>
@@ -1573,10 +1591,10 @@
     <t>Verify language selection dropdown is present and operable.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:29.310Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:30.764Z</t>
+    <t>2026-06-14T11:40:45.370Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:46.774Z</t>
   </si>
   <si>
     <t>TC-100</t>
@@ -1588,10 +1606,10 @@
     <t>Click "Sign Out" and verify browser is redirected back to /login.</t>
   </si>
   <si>
-    <t>2026-06-13T04:30:29.342Z</t>
-  </si>
-  <si>
-    <t>2026-06-13T04:30:30.266Z</t>
+    <t>2026-06-14T11:40:45.407Z</t>
+  </si>
+  <si>
+    <t>2026-06-14T11:40:46.760Z</t>
   </si>
 </sst>
 </file>
@@ -2357,7 +2375,7 @@
         <v>27</v>
       </c>
       <c r="H9" s="20">
-        <v>1152</v>
+        <v>1661</v>
       </c>
       <c r="I9" s="18" t="s">
         <v>28</v>
@@ -2386,7 +2404,7 @@
         <v>33</v>
       </c>
       <c r="H10" s="23">
-        <v>1280</v>
+        <v>1730</v>
       </c>
       <c r="I10" s="22" t="s">
         <v>28</v>
@@ -2415,7 +2433,7 @@
         <v>38</v>
       </c>
       <c r="H11" s="20">
-        <v>1455</v>
+        <v>735</v>
       </c>
       <c r="I11" s="18" t="s">
         <v>28</v>
@@ -2444,7 +2462,7 @@
         <v>43</v>
       </c>
       <c r="H12" s="23">
-        <v>733</v>
+        <v>1640</v>
       </c>
       <c r="I12" s="22" t="s">
         <v>28</v>
@@ -2473,7 +2491,7 @@
         <v>48</v>
       </c>
       <c r="H13" s="20">
-        <v>1568</v>
+        <v>438</v>
       </c>
       <c r="I13" s="18" t="s">
         <v>28</v>
@@ -2502,7 +2520,7 @@
         <v>53</v>
       </c>
       <c r="H14" s="23">
-        <v>500</v>
+        <v>656</v>
       </c>
       <c r="I14" s="22" t="s">
         <v>28</v>
@@ -2531,7 +2549,7 @@
         <v>58</v>
       </c>
       <c r="H15" s="20">
-        <v>1514</v>
+        <v>1239</v>
       </c>
       <c r="I15" s="18" t="s">
         <v>28</v>
@@ -2560,7 +2578,7 @@
         <v>63</v>
       </c>
       <c r="H16" s="23">
-        <v>1026</v>
+        <v>756</v>
       </c>
       <c r="I16" s="22" t="s">
         <v>28</v>
@@ -2589,7 +2607,7 @@
         <v>68</v>
       </c>
       <c r="H17" s="20">
-        <v>904</v>
+        <v>760</v>
       </c>
       <c r="I17" s="18" t="s">
         <v>28</v>
@@ -2618,7 +2636,7 @@
         <v>73</v>
       </c>
       <c r="H18" s="23">
-        <v>475</v>
+        <v>1425</v>
       </c>
       <c r="I18" s="22" t="s">
         <v>28</v>
@@ -2647,7 +2665,7 @@
         <v>79</v>
       </c>
       <c r="H19" s="20">
-        <v>1579</v>
+        <v>999</v>
       </c>
       <c r="I19" s="18" t="s">
         <v>28</v>
@@ -2676,7 +2694,7 @@
         <v>84</v>
       </c>
       <c r="H20" s="23">
-        <v>410</v>
+        <v>1330</v>
       </c>
       <c r="I20" s="22" t="s">
         <v>28</v>
@@ -2705,7 +2723,7 @@
         <v>89</v>
       </c>
       <c r="H21" s="20">
-        <v>1004</v>
+        <v>1250</v>
       </c>
       <c r="I21" s="18" t="s">
         <v>28</v>
@@ -2734,7 +2752,7 @@
         <v>94</v>
       </c>
       <c r="H22" s="23">
-        <v>1203</v>
+        <v>623</v>
       </c>
       <c r="I22" s="22" t="s">
         <v>28</v>
@@ -2763,7 +2781,7 @@
         <v>99</v>
       </c>
       <c r="H23" s="20">
-        <v>827</v>
+        <v>667</v>
       </c>
       <c r="I23" s="18" t="s">
         <v>28</v>
@@ -2792,7 +2810,7 @@
         <v>104</v>
       </c>
       <c r="H24" s="23">
-        <v>629</v>
+        <v>366</v>
       </c>
       <c r="I24" s="22" t="s">
         <v>28</v>
@@ -2821,7 +2839,7 @@
         <v>109</v>
       </c>
       <c r="H25" s="20">
-        <v>1283</v>
+        <v>1548</v>
       </c>
       <c r="I25" s="18" t="s">
         <v>28</v>
@@ -2850,7 +2868,7 @@
         <v>114</v>
       </c>
       <c r="H26" s="23">
-        <v>1131</v>
+        <v>1418</v>
       </c>
       <c r="I26" s="22" t="s">
         <v>28</v>
@@ -2879,7 +2897,7 @@
         <v>119</v>
       </c>
       <c r="H27" s="20">
-        <v>1074</v>
+        <v>988</v>
       </c>
       <c r="I27" s="18" t="s">
         <v>28</v>
@@ -2908,7 +2926,7 @@
         <v>124</v>
       </c>
       <c r="H28" s="23">
-        <v>1558</v>
+        <v>1522</v>
       </c>
       <c r="I28" s="22" t="s">
         <v>28</v>
@@ -2937,7 +2955,7 @@
         <v>129</v>
       </c>
       <c r="H29" s="20">
-        <v>1217</v>
+        <v>1211</v>
       </c>
       <c r="I29" s="18" t="s">
         <v>28</v>
@@ -2966,7 +2984,7 @@
         <v>134</v>
       </c>
       <c r="H30" s="23">
-        <v>1605</v>
+        <v>1035</v>
       </c>
       <c r="I30" s="22" t="s">
         <v>28</v>
@@ -2995,7 +3013,7 @@
         <v>139</v>
       </c>
       <c r="H31" s="20">
-        <v>494</v>
+        <v>1159</v>
       </c>
       <c r="I31" s="18" t="s">
         <v>28</v>
@@ -3024,7 +3042,7 @@
         <v>144</v>
       </c>
       <c r="H32" s="23">
-        <v>1514</v>
+        <v>825</v>
       </c>
       <c r="I32" s="22" t="s">
         <v>28</v>
@@ -3053,7 +3071,7 @@
         <v>150</v>
       </c>
       <c r="H33" s="20">
-        <v>1411</v>
+        <v>1218</v>
       </c>
       <c r="I33" s="18" t="s">
         <v>28</v>
@@ -3082,7 +3100,7 @@
         <v>155</v>
       </c>
       <c r="H34" s="23">
-        <v>566</v>
+        <v>1705</v>
       </c>
       <c r="I34" s="22" t="s">
         <v>28</v>
@@ -3111,7 +3129,7 @@
         <v>160</v>
       </c>
       <c r="H35" s="20">
-        <v>1668</v>
+        <v>1561</v>
       </c>
       <c r="I35" s="18" t="s">
         <v>28</v>
@@ -3140,7 +3158,7 @@
         <v>165</v>
       </c>
       <c r="H36" s="23">
-        <v>845</v>
+        <v>527</v>
       </c>
       <c r="I36" s="22" t="s">
         <v>28</v>
@@ -3166,10 +3184,10 @@
         <v>170</v>
       </c>
       <c r="G37" s="18" t="s">
-        <v>38</v>
+        <v>171</v>
       </c>
       <c r="H37" s="20">
-        <v>492</v>
+        <v>1702</v>
       </c>
       <c r="I37" s="18" t="s">
         <v>28</v>
@@ -3177,28 +3195,28 @@
     </row>
     <row r="38" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="21" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B38" s="22" t="s">
         <v>167</v>
       </c>
       <c r="C38" s="22" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D38" s="22" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E38" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F38" s="22" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="G38" s="22" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H38" s="23">
-        <v>516</v>
+        <v>1274</v>
       </c>
       <c r="I38" s="22" t="s">
         <v>28</v>
@@ -3206,28 +3224,28 @@
     </row>
     <row r="39" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="17" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B39" s="18" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C39" s="18" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D39" s="18" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="E39" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F39" s="18" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="G39" s="18" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
       <c r="H39" s="20">
-        <v>482</v>
+        <v>511</v>
       </c>
       <c r="I39" s="18" t="s">
         <v>28</v>
@@ -3235,28 +3253,28 @@
     </row>
     <row r="40" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="21" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B40" s="22" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C40" s="22" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="D40" s="22" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="E40" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F40" s="22" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="G40" s="22" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="H40" s="23">
-        <v>1635</v>
+        <v>1403</v>
       </c>
       <c r="I40" s="22" t="s">
         <v>28</v>
@@ -3264,28 +3282,28 @@
     </row>
     <row r="41" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="17" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B41" s="18" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C41" s="18" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="D41" s="18" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="E41" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F41" s="18" t="s">
-        <v>189</v>
+        <v>99</v>
       </c>
       <c r="G41" s="18" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="H41" s="20">
-        <v>1620</v>
+        <v>1404</v>
       </c>
       <c r="I41" s="18" t="s">
         <v>28</v>
@@ -3293,28 +3311,28 @@
     </row>
     <row r="42" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="21" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B42" s="22" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C42" s="22" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D42" s="22" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E42" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F42" s="22" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="G42" s="22" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="H42" s="23">
-        <v>465</v>
+        <v>431</v>
       </c>
       <c r="I42" s="22" t="s">
         <v>28</v>
@@ -3322,28 +3340,28 @@
     </row>
     <row r="43" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="17" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B43" s="18" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C43" s="18" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D43" s="18" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E43" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F43" s="18" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="G43" s="18" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="H43" s="20">
-        <v>973</v>
+        <v>1718</v>
       </c>
       <c r="I43" s="18" t="s">
         <v>28</v>
@@ -3351,28 +3369,28 @@
     </row>
     <row r="44" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="21" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B44" s="22" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C44" s="22" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D44" s="22" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="E44" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F44" s="22" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="G44" s="22" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="H44" s="23">
-        <v>1717</v>
+        <v>736</v>
       </c>
       <c r="I44" s="22" t="s">
         <v>28</v>
@@ -3380,28 +3398,28 @@
     </row>
     <row r="45" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="17" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B45" s="18" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C45" s="18" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D45" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="E45" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F45" s="18" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G45" s="18" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="H45" s="20">
-        <v>920</v>
+        <v>393</v>
       </c>
       <c r="I45" s="18" t="s">
         <v>28</v>
@@ -3409,28 +3427,28 @@
     </row>
     <row r="46" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="21" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B46" s="22" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C46" s="22" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D46" s="22" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E46" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F46" s="22" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="G46" s="22" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="H46" s="23">
-        <v>1468</v>
+        <v>407</v>
       </c>
       <c r="I46" s="22" t="s">
         <v>28</v>
@@ -3438,28 +3456,28 @@
     </row>
     <row r="47" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="17" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B47" s="18" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C47" s="18" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D47" s="18" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E47" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F47" s="18" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="G47" s="18" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="H47" s="20">
-        <v>832</v>
+        <v>702</v>
       </c>
       <c r="I47" s="18" t="s">
         <v>28</v>
@@ -3467,28 +3485,28 @@
     </row>
     <row r="48" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="21" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B48" s="22" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C48" s="22" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D48" s="22" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E48" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F48" s="22" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="G48" s="22" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="H48" s="23">
-        <v>1640</v>
+        <v>1111</v>
       </c>
       <c r="I48" s="22" t="s">
         <v>28</v>
@@ -3496,28 +3514,28 @@
     </row>
     <row r="49" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" s="17" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B49" s="18" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C49" s="18" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D49" s="18" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E49" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F49" s="18" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="G49" s="18" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="H49" s="20">
-        <v>417</v>
+        <v>1426</v>
       </c>
       <c r="I49" s="18" t="s">
         <v>28</v>
@@ -3525,28 +3543,28 @@
     </row>
     <row r="50" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="21" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B50" s="22" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C50" s="22" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D50" s="22" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E50" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F50" s="22" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G50" s="22" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="H50" s="23">
-        <v>1441</v>
+        <v>1585</v>
       </c>
       <c r="I50" s="22" t="s">
         <v>28</v>
@@ -3554,28 +3572,28 @@
     </row>
     <row r="51" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" s="17" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B51" s="18" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C51" s="18" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D51" s="18" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E51" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F51" s="18" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="G51" s="18" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="H51" s="20">
-        <v>1015</v>
+        <v>498</v>
       </c>
       <c r="I51" s="18" t="s">
         <v>28</v>
@@ -3583,28 +3601,28 @@
     </row>
     <row r="52" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="21" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B52" s="22" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C52" s="22" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D52" s="22" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="E52" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F52" s="22" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="G52" s="22" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="H52" s="23">
-        <v>1109</v>
+        <v>381</v>
       </c>
       <c r="I52" s="22" t="s">
         <v>28</v>
@@ -3612,28 +3630,28 @@
     </row>
     <row r="53" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" s="17" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B53" s="18" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C53" s="18" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D53" s="18" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E53" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F53" s="18" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="G53" s="18" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="H53" s="20">
-        <v>469</v>
+        <v>743</v>
       </c>
       <c r="I53" s="18" t="s">
         <v>28</v>
@@ -3641,28 +3659,28 @@
     </row>
     <row r="54" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" s="21" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B54" s="22" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C54" s="22" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D54" s="22" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E54" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F54" s="22" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="G54" s="22" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="H54" s="23">
-        <v>1255</v>
+        <v>1121</v>
       </c>
       <c r="I54" s="22" t="s">
         <v>28</v>
@@ -3670,28 +3688,28 @@
     </row>
     <row r="55" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" s="17" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B55" s="18" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C55" s="18" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D55" s="18" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E55" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F55" s="18" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="G55" s="18" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="H55" s="20">
-        <v>529</v>
+        <v>660</v>
       </c>
       <c r="I55" s="18" t="s">
         <v>28</v>
@@ -3699,28 +3717,28 @@
     </row>
     <row r="56" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" s="21" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B56" s="22" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C56" s="22" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D56" s="22" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="E56" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F56" s="22" t="s">
-        <v>119</v>
+        <v>266</v>
       </c>
       <c r="G56" s="22" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="H56" s="23">
-        <v>1519</v>
+        <v>1481</v>
       </c>
       <c r="I56" s="22" t="s">
         <v>28</v>
@@ -3728,28 +3746,28 @@
     </row>
     <row r="57" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" s="17" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B57" s="18" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C57" s="18" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="D57" s="18" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="E57" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F57" s="18" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="G57" s="18" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="H57" s="20">
-        <v>836</v>
+        <v>1067</v>
       </c>
       <c r="I57" s="18" t="s">
         <v>28</v>
@@ -3757,28 +3775,28 @@
     </row>
     <row r="58" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" s="21" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B58" s="22" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C58" s="22" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="D58" s="22" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="E58" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F58" s="22" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="G58" s="22" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="H58" s="23">
-        <v>1370</v>
+        <v>1244</v>
       </c>
       <c r="I58" s="22" t="s">
         <v>28</v>
@@ -3786,28 +3804,28 @@
     </row>
     <row r="59" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" s="17" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B59" s="18" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C59" s="18" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="D59" s="18" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="E59" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F59" s="18" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="G59" s="18" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="H59" s="20">
-        <v>950</v>
+        <v>852</v>
       </c>
       <c r="I59" s="18" t="s">
         <v>28</v>
@@ -3815,28 +3833,28 @@
     </row>
     <row r="60" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" s="21" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B60" s="22" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C60" s="22" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="D60" s="22" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="E60" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F60" s="22" t="s">
-        <v>230</v>
+        <v>286</v>
       </c>
       <c r="G60" s="22" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="H60" s="23">
-        <v>1387</v>
+        <v>478</v>
       </c>
       <c r="I60" s="22" t="s">
         <v>28</v>
@@ -3844,28 +3862,28 @@
     </row>
     <row r="61" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" s="17" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="B61" s="18" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C61" s="18" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="D61" s="18" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="E61" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F61" s="18" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="G61" s="18" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="H61" s="20">
-        <v>623</v>
+        <v>898</v>
       </c>
       <c r="I61" s="18" t="s">
         <v>28</v>
@@ -3873,28 +3891,28 @@
     </row>
     <row r="62" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" s="21" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="B62" s="22" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C62" s="22" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="D62" s="22" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="E62" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F62" s="22" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="G62" s="22" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="H62" s="23">
-        <v>1151</v>
+        <v>834</v>
       </c>
       <c r="I62" s="22" t="s">
         <v>28</v>
@@ -3902,28 +3920,28 @@
     </row>
     <row r="63" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" s="17" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="B63" s="18" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C63" s="18" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="D63" s="18" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="E63" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F63" s="18" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="G63" s="18" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="H63" s="20">
-        <v>626</v>
+        <v>1593</v>
       </c>
       <c r="I63" s="18" t="s">
         <v>28</v>
@@ -3931,28 +3949,28 @@
     </row>
     <row r="64" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" s="21" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="B64" s="22" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C64" s="22" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="D64" s="22" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="E64" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F64" s="22" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="G64" s="22" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="H64" s="23">
-        <v>418</v>
+        <v>1679</v>
       </c>
       <c r="I64" s="22" t="s">
         <v>28</v>
@@ -3960,28 +3978,28 @@
     </row>
     <row r="65" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" s="17" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="B65" s="18" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C65" s="18" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="D65" s="18" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="E65" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F65" s="18" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="G65" s="18" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="H65" s="20">
-        <v>1308</v>
+        <v>377</v>
       </c>
       <c r="I65" s="18" t="s">
         <v>28</v>
@@ -3989,28 +4007,28 @@
     </row>
     <row r="66" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" s="21" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="B66" s="22" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C66" s="22" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="D66" s="22" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="E66" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F66" s="22" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="G66" s="22" t="s">
-        <v>185</v>
+        <v>317</v>
       </c>
       <c r="H66" s="23">
-        <v>664</v>
+        <v>1115</v>
       </c>
       <c r="I66" s="22" t="s">
         <v>28</v>
@@ -4018,28 +4036,28 @@
     </row>
     <row r="67" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" s="17" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="B67" s="18" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C67" s="18" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
       <c r="D67" s="18" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="E67" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F67" s="18" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="G67" s="18" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
       <c r="H67" s="20">
-        <v>358</v>
+        <v>988</v>
       </c>
       <c r="I67" s="18" t="s">
         <v>28</v>
@@ -4047,28 +4065,28 @@
     </row>
     <row r="68" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68" s="21" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
       <c r="B68" s="22" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C68" s="22" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
       <c r="D68" s="22" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
       <c r="E68" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F68" s="22" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="G68" s="22" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="H68" s="23">
-        <v>731</v>
+        <v>1499</v>
       </c>
       <c r="I68" s="22" t="s">
         <v>28</v>
@@ -4076,28 +4094,28 @@
     </row>
     <row r="69" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" s="17" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="B69" s="18" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="C69" s="18" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="D69" s="18" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="E69" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F69" s="18" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="G69" s="18" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="H69" s="20">
-        <v>680</v>
+        <v>1591</v>
       </c>
       <c r="I69" s="18" t="s">
         <v>28</v>
@@ -4105,28 +4123,28 @@
     </row>
     <row r="70" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" s="21" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="B70" s="22" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="C70" s="22" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
       <c r="D70" s="22" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="E70" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F70" s="22" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="G70" s="22" t="s">
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="H70" s="23">
-        <v>1499</v>
+        <v>1520</v>
       </c>
       <c r="I70" s="22" t="s">
         <v>28</v>
@@ -4134,28 +4152,28 @@
     </row>
     <row r="71" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" s="17" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="B71" s="18" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="C71" s="18" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="D71" s="18" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="E71" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F71" s="18" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="G71" s="18" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="H71" s="20">
-        <v>1366</v>
+        <v>635</v>
       </c>
       <c r="I71" s="18" t="s">
         <v>28</v>
@@ -4163,28 +4181,28 @@
     </row>
     <row r="72" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" s="21" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="B72" s="22" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="C72" s="22" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="D72" s="22" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="E72" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F72" s="22" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
       <c r="G72" s="22" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="H72" s="23">
-        <v>1570</v>
+        <v>965</v>
       </c>
       <c r="I72" s="22" t="s">
         <v>28</v>
@@ -4192,28 +4210,28 @@
     </row>
     <row r="73" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" s="17" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="B73" s="18" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="C73" s="18" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="D73" s="18" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="E73" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F73" s="18" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="G73" s="18" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
       <c r="H73" s="20">
-        <v>351</v>
+        <v>1668</v>
       </c>
       <c r="I73" s="18" t="s">
         <v>28</v>
@@ -4221,28 +4239,28 @@
     </row>
     <row r="74" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" s="21" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="B74" s="22" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="C74" s="22" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
       <c r="D74" s="22" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="E74" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F74" s="22" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="G74" s="22" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="H74" s="23">
-        <v>1038</v>
+        <v>1556</v>
       </c>
       <c r="I74" s="22" t="s">
         <v>28</v>
@@ -4250,28 +4268,28 @@
     </row>
     <row r="75" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75" s="17" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="B75" s="18" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="C75" s="18" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="D75" s="18" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="E75" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F75" s="18" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="G75" s="18" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
       <c r="H75" s="20">
-        <v>946</v>
+        <v>1470</v>
       </c>
       <c r="I75" s="18" t="s">
         <v>28</v>
@@ -4279,28 +4297,28 @@
     </row>
     <row r="76" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76" s="21" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="B76" s="22" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="C76" s="22" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="D76" s="22" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="E76" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F76" s="22" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="G76" s="22" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="H76" s="23">
-        <v>1702</v>
+        <v>476</v>
       </c>
       <c r="I76" s="22" t="s">
         <v>28</v>
@@ -4308,28 +4326,28 @@
     </row>
     <row r="77" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77" s="17" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="B77" s="18" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="C77" s="18" t="s">
-        <v>366</v>
+        <v>370</v>
       </c>
       <c r="D77" s="18" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="E77" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F77" s="18" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="G77" s="18" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="H77" s="20">
-        <v>1197</v>
+        <v>742</v>
       </c>
       <c r="I77" s="18" t="s">
         <v>28</v>
@@ -4337,28 +4355,28 @@
     </row>
     <row r="78" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78" s="21" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="B78" s="22" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="C78" s="22" t="s">
-        <v>371</v>
+        <v>375</v>
       </c>
       <c r="D78" s="22" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="E78" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F78" s="22" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
       <c r="G78" s="22" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="H78" s="23">
-        <v>618</v>
+        <v>489</v>
       </c>
       <c r="I78" s="22" t="s">
         <v>28</v>
@@ -4366,28 +4384,28 @@
     </row>
     <row r="79" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79" s="17" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
       <c r="B79" s="18" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="C79" s="18" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
       <c r="D79" s="18" t="s">
-        <v>377</v>
+        <v>381</v>
       </c>
       <c r="E79" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F79" s="18" t="s">
-        <v>378</v>
+        <v>382</v>
       </c>
       <c r="G79" s="18" t="s">
-        <v>379</v>
+        <v>383</v>
       </c>
       <c r="H79" s="20">
-        <v>1225</v>
+        <v>352</v>
       </c>
       <c r="I79" s="18" t="s">
         <v>28</v>
@@ -4395,28 +4413,28 @@
     </row>
     <row r="80" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80" s="21" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="B80" s="22" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="C80" s="22" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
       <c r="D80" s="22" t="s">
-        <v>382</v>
+        <v>386</v>
       </c>
       <c r="E80" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F80" s="22" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="G80" s="22" t="s">
-        <v>384</v>
+        <v>388</v>
       </c>
       <c r="H80" s="23">
-        <v>851</v>
+        <v>1355</v>
       </c>
       <c r="I80" s="22" t="s">
         <v>28</v>
@@ -4424,28 +4442,28 @@
     </row>
     <row r="81" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A81" s="17" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="B81" s="18" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="C81" s="18" t="s">
-        <v>387</v>
+        <v>391</v>
       </c>
       <c r="D81" s="18" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="E81" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F81" s="18" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
       <c r="G81" s="18" t="s">
-        <v>390</v>
+        <v>394</v>
       </c>
       <c r="H81" s="20">
-        <v>1299</v>
+        <v>501</v>
       </c>
       <c r="I81" s="18" t="s">
         <v>28</v>
@@ -4453,28 +4471,28 @@
     </row>
     <row r="82" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82" s="21" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
       <c r="B82" s="22" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="C82" s="22" t="s">
-        <v>392</v>
+        <v>396</v>
       </c>
       <c r="D82" s="22" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="E82" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F82" s="22" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="G82" s="22" t="s">
-        <v>395</v>
+        <v>399</v>
       </c>
       <c r="H82" s="23">
-        <v>576</v>
+        <v>1174</v>
       </c>
       <c r="I82" s="22" t="s">
         <v>28</v>
@@ -4482,28 +4500,28 @@
     </row>
     <row r="83" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" s="17" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="B83" s="18" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="C83" s="18" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="D83" s="18" t="s">
-        <v>398</v>
+        <v>402</v>
       </c>
       <c r="E83" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F83" s="18" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
       <c r="G83" s="18" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
       <c r="H83" s="20">
-        <v>1005</v>
+        <v>822</v>
       </c>
       <c r="I83" s="18" t="s">
         <v>28</v>
@@ -4511,28 +4529,28 @@
     </row>
     <row r="84" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84" s="21" t="s">
-        <v>401</v>
+        <v>405</v>
       </c>
       <c r="B84" s="22" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="C84" s="22" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="D84" s="22" t="s">
-        <v>403</v>
+        <v>407</v>
       </c>
       <c r="E84" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F84" s="22" t="s">
-        <v>404</v>
+        <v>408</v>
       </c>
       <c r="G84" s="22" t="s">
-        <v>405</v>
+        <v>409</v>
       </c>
       <c r="H84" s="23">
-        <v>399</v>
+        <v>596</v>
       </c>
       <c r="I84" s="22" t="s">
         <v>28</v>
@@ -4540,28 +4558,28 @@
     </row>
     <row r="85" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85" s="17" t="s">
-        <v>406</v>
+        <v>410</v>
       </c>
       <c r="B85" s="18" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="C85" s="18" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="D85" s="18" t="s">
-        <v>408</v>
+        <v>412</v>
       </c>
       <c r="E85" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F85" s="18" t="s">
-        <v>409</v>
+        <v>413</v>
       </c>
       <c r="G85" s="18" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="H85" s="20">
-        <v>1599</v>
+        <v>985</v>
       </c>
       <c r="I85" s="18" t="s">
         <v>28</v>
@@ -4569,28 +4587,28 @@
     </row>
     <row r="86" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86" s="21" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="B86" s="22" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="C86" s="22" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="D86" s="22" t="s">
-        <v>413</v>
+        <v>417</v>
       </c>
       <c r="E86" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F86" s="22" t="s">
-        <v>414</v>
+        <v>418</v>
       </c>
       <c r="G86" s="22" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="H86" s="23">
-        <v>1052</v>
+        <v>397</v>
       </c>
       <c r="I86" s="22" t="s">
         <v>28</v>
@@ -4598,28 +4616,28 @@
     </row>
     <row r="87" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87" s="17" t="s">
-        <v>416</v>
+        <v>420</v>
       </c>
       <c r="B87" s="18" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="C87" s="18" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
       <c r="D87" s="18" t="s">
-        <v>418</v>
+        <v>422</v>
       </c>
       <c r="E87" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F87" s="18" t="s">
-        <v>419</v>
+        <v>423</v>
       </c>
       <c r="G87" s="18" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="H87" s="20">
-        <v>1470</v>
+        <v>469</v>
       </c>
       <c r="I87" s="18" t="s">
         <v>28</v>
@@ -4627,28 +4645,28 @@
     </row>
     <row r="88" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88" s="21" t="s">
-        <v>421</v>
+        <v>425</v>
       </c>
       <c r="B88" s="22" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="C88" s="22" t="s">
-        <v>422</v>
+        <v>426</v>
       </c>
       <c r="D88" s="22" t="s">
-        <v>423</v>
+        <v>427</v>
       </c>
       <c r="E88" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F88" s="22" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="G88" s="22" t="s">
-        <v>425</v>
+        <v>429</v>
       </c>
       <c r="H88" s="23">
-        <v>1314</v>
+        <v>413</v>
       </c>
       <c r="I88" s="22" t="s">
         <v>28</v>
@@ -4656,28 +4674,28 @@
     </row>
     <row r="89" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89" s="17" t="s">
-        <v>426</v>
+        <v>430</v>
       </c>
       <c r="B89" s="18" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="C89" s="18" t="s">
-        <v>427</v>
+        <v>431</v>
       </c>
       <c r="D89" s="18" t="s">
-        <v>428</v>
+        <v>432</v>
       </c>
       <c r="E89" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F89" s="18" t="s">
-        <v>429</v>
+        <v>433</v>
       </c>
       <c r="G89" s="18" t="s">
-        <v>430</v>
+        <v>434</v>
       </c>
       <c r="H89" s="20">
-        <v>1603</v>
+        <v>1601</v>
       </c>
       <c r="I89" s="18" t="s">
         <v>28</v>
@@ -4685,28 +4703,28 @@
     </row>
     <row r="90" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90" s="21" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
       <c r="B90" s="22" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="C90" s="22" t="s">
-        <v>432</v>
+        <v>436</v>
       </c>
       <c r="D90" s="22" t="s">
-        <v>433</v>
+        <v>437</v>
       </c>
       <c r="E90" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F90" s="22" t="s">
-        <v>434</v>
+        <v>438</v>
       </c>
       <c r="G90" s="22" t="s">
-        <v>435</v>
+        <v>439</v>
       </c>
       <c r="H90" s="23">
-        <v>1169</v>
+        <v>947</v>
       </c>
       <c r="I90" s="22" t="s">
         <v>28</v>
@@ -4714,28 +4732,28 @@
     </row>
     <row r="91" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91" s="17" t="s">
-        <v>436</v>
+        <v>440</v>
       </c>
       <c r="B91" s="18" t="s">
-        <v>437</v>
+        <v>441</v>
       </c>
       <c r="C91" s="18" t="s">
-        <v>438</v>
+        <v>442</v>
       </c>
       <c r="D91" s="18" t="s">
-        <v>439</v>
+        <v>443</v>
       </c>
       <c r="E91" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F91" s="18" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
       <c r="G91" s="18" t="s">
-        <v>441</v>
+        <v>445</v>
       </c>
       <c r="H91" s="20">
-        <v>1004</v>
+        <v>565</v>
       </c>
       <c r="I91" s="18" t="s">
         <v>28</v>
@@ -4743,25 +4761,25 @@
     </row>
     <row r="92" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92" s="21" t="s">
-        <v>442</v>
+        <v>446</v>
       </c>
       <c r="B92" s="22" t="s">
-        <v>437</v>
+        <v>441</v>
       </c>
       <c r="C92" s="22" t="s">
-        <v>443</v>
+        <v>447</v>
       </c>
       <c r="D92" s="22" t="s">
-        <v>444</v>
+        <v>448</v>
       </c>
       <c r="E92" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F92" s="22" t="s">
-        <v>225</v>
+        <v>449</v>
       </c>
       <c r="G92" s="22" t="s">
-        <v>445</v>
+        <v>450</v>
       </c>
       <c r="H92" s="23">
         <v>1444</v>
@@ -4772,28 +4790,28 @@
     </row>
     <row r="93" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A93" s="17" t="s">
-        <v>446</v>
+        <v>451</v>
       </c>
       <c r="B93" s="18" t="s">
-        <v>437</v>
+        <v>441</v>
       </c>
       <c r="C93" s="18" t="s">
-        <v>447</v>
+        <v>452</v>
       </c>
       <c r="D93" s="18" t="s">
-        <v>448</v>
+        <v>453</v>
       </c>
       <c r="E93" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F93" s="18" t="s">
-        <v>449</v>
+        <v>454</v>
       </c>
       <c r="G93" s="18" t="s">
-        <v>450</v>
+        <v>455</v>
       </c>
       <c r="H93" s="20">
-        <v>468</v>
+        <v>824</v>
       </c>
       <c r="I93" s="18" t="s">
         <v>28</v>
@@ -4801,28 +4819,28 @@
     </row>
     <row r="94" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A94" s="21" t="s">
-        <v>451</v>
+        <v>456</v>
       </c>
       <c r="B94" s="22" t="s">
-        <v>437</v>
+        <v>441</v>
       </c>
       <c r="C94" s="22" t="s">
-        <v>452</v>
+        <v>457</v>
       </c>
       <c r="D94" s="22" t="s">
-        <v>453</v>
+        <v>458</v>
       </c>
       <c r="E94" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F94" s="22" t="s">
-        <v>454</v>
+        <v>459</v>
       </c>
       <c r="G94" s="22" t="s">
-        <v>455</v>
+        <v>460</v>
       </c>
       <c r="H94" s="23">
-        <v>364</v>
+        <v>356</v>
       </c>
       <c r="I94" s="22" t="s">
         <v>28</v>
@@ -4830,28 +4848,28 @@
     </row>
     <row r="95" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A95" s="17" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="B95" s="18" t="s">
-        <v>457</v>
+        <v>462</v>
       </c>
       <c r="C95" s="18" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="D95" s="18" t="s">
-        <v>459</v>
+        <v>464</v>
       </c>
       <c r="E95" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F95" s="18" t="s">
-        <v>460</v>
+        <v>465</v>
       </c>
       <c r="G95" s="18" t="s">
-        <v>461</v>
+        <v>466</v>
       </c>
       <c r="H95" s="20">
-        <v>1002</v>
+        <v>1548</v>
       </c>
       <c r="I95" s="18" t="s">
         <v>28</v>
@@ -4859,28 +4877,28 @@
     </row>
     <row r="96" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A96" s="21" t="s">
+        <v>467</v>
+      </c>
+      <c r="B96" s="22" t="s">
         <v>462</v>
       </c>
-      <c r="B96" s="22" t="s">
-        <v>457</v>
-      </c>
       <c r="C96" s="22" t="s">
-        <v>463</v>
+        <v>468</v>
       </c>
       <c r="D96" s="22" t="s">
-        <v>464</v>
+        <v>469</v>
       </c>
       <c r="E96" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F96" s="22" t="s">
-        <v>465</v>
+        <v>470</v>
       </c>
       <c r="G96" s="22" t="s">
-        <v>466</v>
+        <v>471</v>
       </c>
       <c r="H96" s="23">
-        <v>600</v>
+        <v>868</v>
       </c>
       <c r="I96" s="22" t="s">
         <v>28</v>
@@ -4888,28 +4906,28 @@
     </row>
     <row r="97" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A97" s="17" t="s">
-        <v>467</v>
+        <v>472</v>
       </c>
       <c r="B97" s="18" t="s">
-        <v>457</v>
+        <v>462</v>
       </c>
       <c r="C97" s="18" t="s">
-        <v>468</v>
+        <v>473</v>
       </c>
       <c r="D97" s="18" t="s">
-        <v>469</v>
+        <v>474</v>
       </c>
       <c r="E97" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F97" s="18" t="s">
-        <v>470</v>
+        <v>475</v>
       </c>
       <c r="G97" s="18" t="s">
-        <v>471</v>
+        <v>476</v>
       </c>
       <c r="H97" s="20">
-        <v>1003</v>
+        <v>479</v>
       </c>
       <c r="I97" s="18" t="s">
         <v>28</v>
@@ -4917,28 +4935,28 @@
     </row>
     <row r="98" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A98" s="21" t="s">
-        <v>472</v>
+        <v>477</v>
       </c>
       <c r="B98" s="22" t="s">
-        <v>457</v>
+        <v>462</v>
       </c>
       <c r="C98" s="22" t="s">
-        <v>473</v>
+        <v>478</v>
       </c>
       <c r="D98" s="22" t="s">
-        <v>474</v>
+        <v>479</v>
       </c>
       <c r="E98" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F98" s="22" t="s">
-        <v>475</v>
+        <v>480</v>
       </c>
       <c r="G98" s="22" t="s">
-        <v>476</v>
+        <v>481</v>
       </c>
       <c r="H98" s="23">
-        <v>582</v>
+        <v>1176</v>
       </c>
       <c r="I98" s="22" t="s">
         <v>28</v>
@@ -4946,28 +4964,28 @@
     </row>
     <row r="99" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A99" s="17" t="s">
-        <v>477</v>
+        <v>482</v>
       </c>
       <c r="B99" s="18" t="s">
-        <v>457</v>
+        <v>462</v>
       </c>
       <c r="C99" s="18" t="s">
-        <v>478</v>
+        <v>483</v>
       </c>
       <c r="D99" s="18" t="s">
-        <v>479</v>
+        <v>484</v>
       </c>
       <c r="E99" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F99" s="18" t="s">
-        <v>480</v>
+        <v>485</v>
       </c>
       <c r="G99" s="18" t="s">
-        <v>481</v>
+        <v>486</v>
       </c>
       <c r="H99" s="20">
-        <v>670</v>
+        <v>1032</v>
       </c>
       <c r="I99" s="18" t="s">
         <v>28</v>
@@ -4975,28 +4993,28 @@
     </row>
     <row r="100" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100" s="21" t="s">
-        <v>482</v>
+        <v>487</v>
       </c>
       <c r="B100" s="22" t="s">
-        <v>457</v>
+        <v>462</v>
       </c>
       <c r="C100" s="22" t="s">
-        <v>483</v>
+        <v>488</v>
       </c>
       <c r="D100" s="22" t="s">
-        <v>484</v>
+        <v>489</v>
       </c>
       <c r="E100" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F100" s="22" t="s">
-        <v>485</v>
+        <v>490</v>
       </c>
       <c r="G100" s="22" t="s">
-        <v>486</v>
+        <v>491</v>
       </c>
       <c r="H100" s="23">
-        <v>640</v>
+        <v>748</v>
       </c>
       <c r="I100" s="22" t="s">
         <v>28</v>
@@ -5004,28 +5022,28 @@
     </row>
     <row r="101" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101" s="17" t="s">
-        <v>487</v>
+        <v>492</v>
       </c>
       <c r="B101" s="18" t="s">
-        <v>457</v>
+        <v>462</v>
       </c>
       <c r="C101" s="18" t="s">
-        <v>488</v>
+        <v>493</v>
       </c>
       <c r="D101" s="18" t="s">
-        <v>489</v>
+        <v>494</v>
       </c>
       <c r="E101" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F101" s="18" t="s">
-        <v>490</v>
+        <v>495</v>
       </c>
       <c r="G101" s="18" t="s">
-        <v>471</v>
+        <v>496</v>
       </c>
       <c r="H101" s="20">
-        <v>859</v>
+        <v>1588</v>
       </c>
       <c r="I101" s="18" t="s">
         <v>28</v>
@@ -5033,28 +5051,28 @@
     </row>
     <row r="102" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A102" s="21" t="s">
-        <v>491</v>
+        <v>497</v>
       </c>
       <c r="B102" s="22" t="s">
-        <v>457</v>
+        <v>462</v>
       </c>
       <c r="C102" s="22" t="s">
-        <v>492</v>
+        <v>498</v>
       </c>
       <c r="D102" s="22" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E102" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F102" s="22" t="s">
-        <v>494</v>
+        <v>500</v>
       </c>
       <c r="G102" s="22" t="s">
-        <v>495</v>
+        <v>501</v>
       </c>
       <c r="H102" s="23">
-        <v>824</v>
+        <v>1357</v>
       </c>
       <c r="I102" s="22" t="s">
         <v>28</v>
@@ -5062,28 +5080,28 @@
     </row>
     <row r="103" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A103" s="17" t="s">
-        <v>496</v>
+        <v>502</v>
       </c>
       <c r="B103" s="18" t="s">
-        <v>497</v>
+        <v>503</v>
       </c>
       <c r="C103" s="18" t="s">
-        <v>498</v>
+        <v>504</v>
       </c>
       <c r="D103" s="18" t="s">
-        <v>499</v>
+        <v>505</v>
       </c>
       <c r="E103" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F103" s="18" t="s">
-        <v>500</v>
+        <v>506</v>
       </c>
       <c r="G103" s="18" t="s">
-        <v>501</v>
+        <v>507</v>
       </c>
       <c r="H103" s="20">
-        <v>1651</v>
+        <v>372</v>
       </c>
       <c r="I103" s="18" t="s">
         <v>28</v>
@@ -5091,28 +5109,28 @@
     </row>
     <row r="104" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A104" s="21" t="s">
-        <v>502</v>
+        <v>508</v>
       </c>
       <c r="B104" s="22" t="s">
-        <v>497</v>
+        <v>503</v>
       </c>
       <c r="C104" s="22" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="D104" s="22" t="s">
-        <v>504</v>
+        <v>510</v>
       </c>
       <c r="E104" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F104" s="22" t="s">
-        <v>505</v>
+        <v>511</v>
       </c>
       <c r="G104" s="22" t="s">
-        <v>506</v>
+        <v>512</v>
       </c>
       <c r="H104" s="23">
-        <v>352</v>
+        <v>1496</v>
       </c>
       <c r="I104" s="22" t="s">
         <v>28</v>
@@ -5120,28 +5138,28 @@
     </row>
     <row r="105" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A105" s="17" t="s">
-        <v>507</v>
+        <v>513</v>
       </c>
       <c r="B105" s="18" t="s">
-        <v>497</v>
+        <v>503</v>
       </c>
       <c r="C105" s="18" t="s">
-        <v>508</v>
+        <v>514</v>
       </c>
       <c r="D105" s="18" t="s">
-        <v>509</v>
+        <v>515</v>
       </c>
       <c r="E105" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F105" s="18" t="s">
-        <v>510</v>
+        <v>516</v>
       </c>
       <c r="G105" s="18" t="s">
-        <v>511</v>
+        <v>517</v>
       </c>
       <c r="H105" s="20">
-        <v>1146</v>
+        <v>1291</v>
       </c>
       <c r="I105" s="18" t="s">
         <v>28</v>
@@ -5149,28 +5167,28 @@
     </row>
     <row r="106" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A106" s="21" t="s">
-        <v>512</v>
+        <v>518</v>
       </c>
       <c r="B106" s="22" t="s">
-        <v>497</v>
+        <v>503</v>
       </c>
       <c r="C106" s="22" t="s">
-        <v>513</v>
+        <v>519</v>
       </c>
       <c r="D106" s="22" t="s">
-        <v>514</v>
+        <v>520</v>
       </c>
       <c r="E106" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F106" s="22" t="s">
-        <v>515</v>
+        <v>521</v>
       </c>
       <c r="G106" s="22" t="s">
-        <v>516</v>
+        <v>522</v>
       </c>
       <c r="H106" s="23">
-        <v>1202</v>
+        <v>1658</v>
       </c>
       <c r="I106" s="22" t="s">
         <v>28</v>
@@ -5178,28 +5196,28 @@
     </row>
     <row r="107" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A107" s="17" t="s">
-        <v>517</v>
+        <v>523</v>
       </c>
       <c r="B107" s="18" t="s">
-        <v>497</v>
+        <v>503</v>
       </c>
       <c r="C107" s="18" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="D107" s="18" t="s">
-        <v>519</v>
+        <v>525</v>
       </c>
       <c r="E107" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F107" s="18" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="G107" s="18" t="s">
-        <v>521</v>
+        <v>527</v>
       </c>
       <c r="H107" s="20">
-        <v>1454</v>
+        <v>1404</v>
       </c>
       <c r="I107" s="18" t="s">
         <v>28</v>
@@ -5207,28 +5225,28 @@
     </row>
     <row r="108" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A108" s="21" t="s">
-        <v>522</v>
+        <v>528</v>
       </c>
       <c r="B108" s="22" t="s">
-        <v>497</v>
+        <v>503</v>
       </c>
       <c r="C108" s="22" t="s">
-        <v>523</v>
+        <v>529</v>
       </c>
       <c r="D108" s="22" t="s">
-        <v>524</v>
+        <v>530</v>
       </c>
       <c r="E108" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F108" s="22" t="s">
-        <v>525</v>
+        <v>531</v>
       </c>
       <c r="G108" s="22" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="H108" s="23">
-        <v>924</v>
+        <v>1353</v>
       </c>
       <c r="I108" s="22" t="s">
         <v>28</v>

</xml_diff>

<commit_message>
feat: dynamic dashboard with Supabase realtime - fix DB column names and data queries
</commit_message>
<xml_diff>
--- a/selenium_tests/reports/selenium_report.xlsx
+++ b/selenium_tests/reports/selenium_report.xlsx
@@ -11,12 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="826" uniqueCount="533">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="826" uniqueCount="528">
   <si>
     <t>VolunteerSync Flutter Web — Selenium E2E Test Report</t>
   </si>
   <si>
-    <t xml:space="preserve">  Browser: Chrome  |  Target: Flutter Web (localhost:8080)  |  Generated: 14/6/2026, 5:10:45 pm</t>
+    <t xml:space="preserve">  Browser: Chrome  |  Target: Flutter Web (localhost:8080)  |  Generated: 20/6/2026, 11:49:45 am</t>
   </si>
   <si>
     <t xml:space="preserve">  EXECUTION SUMMARY</t>
@@ -40,13 +40,13 @@
     <t>Total Duration</t>
   </si>
   <si>
-    <t>103.59s</t>
+    <t>97.21s</t>
   </si>
   <si>
     <t>Run At</t>
   </si>
   <si>
-    <t>14/6/2026, 5:10:45 pm</t>
+    <t>20/6/2026, 11:49:45 am</t>
   </si>
   <si>
     <t>Test ID</t>
@@ -91,10 +91,10 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:41.617Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:43.278Z</t>
+    <t>2026-06-20T06:19:41.794Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:42.470Z</t>
   </si>
   <si>
     <t>No errors. Flow completed successfully.</t>
@@ -109,10 +109,10 @@
     <t>Verify hero section headline text is present and visible on page load.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:41.660Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:43.390Z</t>
+    <t>2026-06-20T06:19:41.839Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:43.380Z</t>
   </si>
   <si>
     <t>TC-003</t>
@@ -124,10 +124,10 @@
     <t>Verify the subtitle/description paragraph appears below the hero title.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:41.699Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:42.434Z</t>
+    <t>2026-06-20T06:19:41.871Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:42.713Z</t>
   </si>
   <si>
     <t>TC-004</t>
@@ -139,10 +139,10 @@
     <t>Verify the gradient VolunteerSync logo/icon is visible in the header.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:41.741Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:43.381Z</t>
+    <t>2026-06-20T06:19:41.901Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:42.921Z</t>
   </si>
   <si>
     <t>TC-005</t>
@@ -154,10 +154,10 @@
     <t>Verify "Get Started" primary CTA button renders and is clickable.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:41.777Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:42.215Z</t>
+    <t>2026-06-20T06:19:41.933Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:42.965Z</t>
   </si>
   <si>
     <t>TC-006</t>
@@ -169,10 +169,10 @@
     <t>Verify clicking "Sign In" navigates the browser to /login route.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:41.818Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:42.474Z</t>
+    <t>2026-06-20T06:19:41.963Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:42.830Z</t>
   </si>
   <si>
     <t>TC-007</t>
@@ -184,10 +184,10 @@
     <t>Verify the features/benefits section is displayed below the hero.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:41.850Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:43.089Z</t>
+    <t>2026-06-20T06:19:42.009Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:42.396Z</t>
   </si>
   <si>
     <t>TC-008</t>
@@ -199,10 +199,10 @@
     <t>Verify numerical statistics blocks (e.g. "1,000+ Volunteers") appear.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:41.882Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:42.638Z</t>
+    <t>2026-06-20T06:19:42.040Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:43.395Z</t>
   </si>
   <si>
     <t>TC-009</t>
@@ -214,10 +214,10 @@
     <t>Verify the browser &lt;title&gt; tag contains "VolunteerSync".</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:41.922Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:42.682Z</t>
+    <t>2026-06-20T06:19:42.072Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:43.110Z</t>
   </si>
   <si>
     <t>TC-010</t>
@@ -229,10 +229,10 @@
     <t>Verify page does not overflow on 1280x900 viewport resolution.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:41.959Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:43.384Z</t>
+    <t>2026-06-20T06:19:42.103Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:43.494Z</t>
   </si>
   <si>
     <t>TC-011</t>
@@ -247,10 +247,10 @@
     <t>Verify /login route loads the login screen without errors.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:41.998Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:42.997Z</t>
+    <t>2026-06-20T06:19:42.134Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:43.833Z</t>
   </si>
   <si>
     <t>TC-012</t>
@@ -262,10 +262,10 @@
     <t>Verify the email input field is rendered and accepts keyboard input.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:42.040Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:43.370Z</t>
+    <t>2026-06-20T06:19:42.165Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:42.842Z</t>
   </si>
   <si>
     <t>TC-013</t>
@@ -277,10 +277,10 @@
     <t>Verify the password field is rendered and masks characters by default.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:42.074Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:43.324Z</t>
+    <t>2026-06-20T06:19:42.196Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:43.152Z</t>
   </si>
   <si>
     <t>TC-014</t>
@@ -292,10 +292,10 @@
     <t>Verify the eye icon toggles the password field to plaintext and back.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:42.116Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:42.739Z</t>
+    <t>2026-06-20T06:19:42.228Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:42.758Z</t>
   </si>
   <si>
     <t>TC-015</t>
@@ -307,10 +307,10 @@
     <t>Verify submitting with no email shows "Enter a valid email" error text.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:42.158Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:42.825Z</t>
+    <t>2026-06-20T06:19:42.259Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:42.779Z</t>
   </si>
   <si>
     <t>TC-016</t>
@@ -322,10 +322,10 @@
     <t>Verify entering "invalidemail" (no @) shows field validation warning.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:42.201Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:42.567Z</t>
+    <t>2026-06-20T06:19:42.290Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:42.877Z</t>
   </si>
   <si>
     <t>TC-017</t>
@@ -337,10 +337,10 @@
     <t>Verify entering a password under 6 characters shows "Min 6 characters".</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:42.241Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:43.789Z</t>
+    <t>2026-06-20T06:19:42.322Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:42.968Z</t>
   </si>
   <si>
     <t>TC-018</t>
@@ -352,10 +352,10 @@
     <t>Verify "Forgot password?" link opens /forgot-password route.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:42.283Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:43.701Z</t>
+    <t>2026-06-20T06:19:42.352Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:43.175Z</t>
   </si>
   <si>
     <t>TC-019</t>
@@ -367,10 +367,10 @@
     <t>Verify "Sign up free →" navigates to /register route.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:42.313Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:43.301Z</t>
+    <t>2026-06-20T06:19:42.383Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:43.200Z</t>
   </si>
   <si>
     <t>TC-020</t>
@@ -382,10 +382,10 @@
     <t>Verify back arrow button returns to the / landing screen.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:42.350Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:43.872Z</t>
+    <t>2026-06-20T06:19:42.414Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:43.293Z</t>
   </si>
   <si>
     <t>TC-021</t>
@@ -397,10 +397,10 @@
     <t>Verify Sign In button transitions to a loading spinner on submit.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:42.383Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:43.594Z</t>
+    <t>2026-06-20T06:19:42.445Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:43.490Z</t>
   </si>
   <si>
     <t>TC-022</t>
@@ -412,10 +412,10 @@
     <t>Verify incorrect credentials show an error banner on the login form.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:42.417Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:43.452Z</t>
+    <t>2026-06-20T06:19:42.476Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:43.407Z</t>
   </si>
   <si>
     <t>TC-023</t>
@@ -427,10 +427,10 @@
     <t>Enter alex@volunteersync.io / password123 and confirm /dashboard redirect.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:42.452Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:43.611Z</t>
+    <t>2026-06-20T06:19:42.507Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:43.065Z</t>
   </si>
   <si>
     <t>TC-024</t>
@@ -442,10 +442,10 @@
     <t>Verify direct navigation to /dashboard redirects to /login if not logged in.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:42.490Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:43.315Z</t>
+    <t>2026-06-20T06:19:42.539Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:44.017Z</t>
   </si>
   <si>
     <t>TC-025</t>
@@ -460,10 +460,10 @@
     <t>Verify /register route renders the onboarding form correctly.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:42.520Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:43.738Z</t>
+    <t>2026-06-20T06:19:42.570Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:43.729Z</t>
   </si>
   <si>
     <t>TC-026</t>
@@ -475,10 +475,10 @@
     <t>Verify Name, Email, Password, and Role fields are present.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:42.560Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:44.265Z</t>
+    <t>2026-06-20T06:19:42.601Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:43.188Z</t>
   </si>
   <si>
     <t>TC-027</t>
@@ -490,10 +490,10 @@
     <t>Verify submitting a blank register form shows required field errors.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:42.599Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:44.160Z</t>
+    <t>2026-06-20T06:19:42.632Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:43.130Z</t>
   </si>
   <si>
     <t>TC-028</t>
@@ -505,10 +505,10 @@
     <t>Verify "Sign in →" link navigates back to /login page.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:42.640Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:43.167Z</t>
+    <t>2026-06-20T06:19:42.665Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:43.670Z</t>
   </si>
   <si>
     <t>TC-029</t>
@@ -523,10 +523,10 @@
     <t>Verify /forgot-password page loads the reset form.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:42.681Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:44.383Z</t>
+    <t>2026-06-20T06:19:42.695Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:44.000Z</t>
   </si>
   <si>
     <t>TC-030</t>
@@ -538,10 +538,10 @@
     <t>Enter email and verify success state screen displays after submit.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:42.725Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:43.999Z</t>
+    <t>2026-06-20T06:19:42.727Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:43.366Z</t>
   </si>
   <si>
     <t>TC-031</t>
@@ -556,10 +556,10 @@
     <t>Verify /dashboard route renders after successful authentication.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:42.758Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:43.269Z</t>
+    <t>2026-06-20T06:19:42.759Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:43.134Z</t>
   </si>
   <si>
     <t>TC-032</t>
@@ -571,10 +571,10 @@
     <t>Verify the left sidebar is displayed with all navigation menu items.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:42.790Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:44.193Z</t>
+    <t>2026-06-20T06:19:42.789Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:43.421Z</t>
   </si>
   <si>
     <t>TC-033</t>
@@ -586,7 +586,10 @@
     <t>Verify the "Total Volunteers" statistic card is present with a number.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:44.229Z</t>
+    <t>2026-06-20T06:19:42.820Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:43.831Z</t>
   </si>
   <si>
     <t>TC-034</t>
@@ -598,10 +601,10 @@
     <t>Verify the "Active Events" KPI card displays correct metric data.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:42.866Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:43.297Z</t>
+    <t>2026-06-20T06:19:42.850Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:43.466Z</t>
   </si>
   <si>
     <t>TC-035</t>
@@ -613,10 +616,10 @@
     <t>Verify the "Total Hours" KPI metric card renders with a number value.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:42.902Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:44.620Z</t>
+    <t>2026-06-20T06:19:42.881Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:43.866Z</t>
   </si>
   <si>
     <t>TC-036</t>
@@ -628,10 +631,10 @@
     <t>Verify the "Retention Rate" percentage card is displayed on dashboard.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:42.936Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:43.672Z</t>
+    <t>2026-06-20T06:19:42.912Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:44.072Z</t>
   </si>
   <si>
     <t>TC-037</t>
@@ -643,10 +646,10 @@
     <t>Verify the line chart rendering the volunteer growth trend is present.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:42.980Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:43.373Z</t>
+    <t>2026-06-20T06:19:42.943Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:44.603Z</t>
   </si>
   <si>
     <t>TC-038</t>
@@ -658,10 +661,10 @@
     <t>Verify the attendance bar chart is rendered with visible columns.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:43.019Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:43.426Z</t>
+    <t>2026-06-20T06:19:42.974Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:44.001Z</t>
   </si>
   <si>
     <t>TC-039</t>
@@ -673,10 +676,10 @@
     <t>Verify the category distribution pie chart is visible on dashboard.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:43.061Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:43.763Z</t>
+    <t>2026-06-20T06:19:43.004Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:44.394Z</t>
   </si>
   <si>
     <t>TC-040</t>
@@ -688,10 +691,10 @@
     <t>Verify the activity feed list shows timestamped volunteer actions.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:43.100Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:44.211Z</t>
+    <t>2026-06-20T06:19:43.036Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:43.739Z</t>
   </si>
   <si>
     <t>TC-041</t>
@@ -703,10 +706,10 @@
     <t>Verify the Volt AI insight recommendation widget is visible.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:43.132Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:44.558Z</t>
+    <t>2026-06-20T06:19:43.067Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:43.827Z</t>
   </si>
   <si>
     <t>TC-042</t>
@@ -718,10 +721,10 @@
     <t>Verify clicking the collapse arrow narrows the sidebar to icon-only mode.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:43.168Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:44.753Z</t>
+    <t>2026-06-20T06:19:43.098Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:44.502Z</t>
   </si>
   <si>
     <t>TC-043</t>
@@ -733,10 +736,7 @@
     <t>Verify clicking the expand icon re-opens the sidebar to full width.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:43.199Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:43.697Z</t>
+    <t>2026-06-20T06:19:44.015Z</t>
   </si>
   <si>
     <t>TC-044</t>
@@ -748,10 +748,10 @@
     <t>Verify the "Dashboard" nav item is highlighted/active on /dashboard.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:43.241Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:43.622Z</t>
+    <t>2026-06-20T06:19:43.161Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:43.878Z</t>
   </si>
   <si>
     <t>TC-045</t>
@@ -763,10 +763,10 @@
     <t>Verify the logged-in user name appears in the sidebar bottom section.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:43.285Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:44.028Z</t>
+    <t>2026-06-20T06:19:43.192Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:43.781Z</t>
   </si>
   <si>
     <t>TC-046</t>
@@ -781,10 +781,10 @@
     <t>Click "Volunteers" in sidebar and verify /volunteers route loads.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:43.331Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:44.452Z</t>
+    <t>2026-06-20T06:19:43.222Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:44.824Z</t>
   </si>
   <si>
     <t>TC-047</t>
@@ -796,10 +796,10 @@
     <t>Verify the volunteer listing grid/list is populated with cards.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:43.366Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:44.026Z</t>
+    <t>2026-06-20T06:19:43.253Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:43.660Z</t>
   </si>
   <si>
     <t>TC-048</t>
@@ -811,10 +811,10 @@
     <t>Verify the search input field is visible and accepts text.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:43.408Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:44.889Z</t>
+    <t>2026-06-20T06:19:43.285Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:44.240Z</t>
   </si>
   <si>
     <t>TC-049</t>
@@ -826,10 +826,10 @@
     <t>Type "Alex" in search and verify filtered results appear.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:43.444Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:44.511Z</t>
+    <t>2026-06-20T06:19:43.316Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:44.232Z</t>
   </si>
   <si>
     <t>TC-050</t>
@@ -841,10 +841,10 @@
     <t>Type "zzznoresult" in search and verify empty state message shows.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:43.490Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:44.734Z</t>
+    <t>2026-06-20T06:19:43.347Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:44.693Z</t>
   </si>
   <si>
     <t>TC-051</t>
@@ -856,10 +856,10 @@
     <t>Click "All" filter chip and verify full volunteer list renders.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:43.532Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:44.384Z</t>
+    <t>2026-06-20T06:19:43.379Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:44.127Z</t>
   </si>
   <si>
     <t>TC-052</t>
@@ -871,10 +871,10 @@
     <t>Click "Active" chip and verify only active volunteers appear.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:43.575Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:44.053Z</t>
+    <t>2026-06-20T06:19:43.411Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:44.963Z</t>
   </si>
   <si>
     <t>TC-053</t>
@@ -886,10 +886,10 @@
     <t>Click "Inactive" chip and verify filtered-down inactive members.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:43.616Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:44.514Z</t>
+    <t>2026-06-20T06:19:43.442Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:44.877Z</t>
   </si>
   <si>
     <t>TC-054</t>
@@ -901,10 +901,10 @@
     <t>Click "Pending" chip and verify pending members list.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:43.653Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:44.487Z</t>
+    <t>2026-06-20T06:19:43.473Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:44.720Z</t>
   </si>
   <si>
     <t>TC-055</t>
@@ -916,10 +916,10 @@
     <t>Verify each volunteer list card shows an avatar with name initials.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:43.696Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:45.289Z</t>
+    <t>2026-06-20T06:19:43.504Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:45.242Z</t>
   </si>
   <si>
     <t>TC-056</t>
@@ -931,10 +931,10 @@
     <t>Click a volunteer card and verify the profile detail sheet slides in.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:43.730Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:45.409Z</t>
+    <t>2026-06-20T06:19:43.535Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:44.046Z</t>
   </si>
   <si>
     <t>TC-057</t>
@@ -946,10 +946,10 @@
     <t>Verify the volunteer email is visible in the opened profile sheet.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:43.764Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:44.141Z</t>
+    <t>2026-06-20T06:19:43.566Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:43.937Z</t>
   </si>
   <si>
     <t>TC-058</t>
@@ -961,10 +961,10 @@
     <t>Verify cumulative hours are listed in the volunteer detail view.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:43.805Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:44.920Z</t>
+    <t>2026-06-20T06:19:43.597Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:44.097Z</t>
   </si>
   <si>
     <t>TC-059</t>
@@ -976,10 +976,10 @@
     <t>Verify team/group badge labels appear in the profile detail sheet.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:43.840Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:44.828Z</t>
+    <t>2026-06-20T06:19:43.627Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:44.478Z</t>
   </si>
   <si>
     <t>TC-060</t>
@@ -991,10 +991,7 @@
     <t>Click outside or close button and verify the profile sheet dismisses.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:43.884Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:45.383Z</t>
+    <t>2026-06-20T06:19:44.451Z</t>
   </si>
   <si>
     <t>TC-061</t>
@@ -1009,10 +1006,10 @@
     <t>Click "Events" sidebar item and verify /events route loads.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:43.915Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:45.506Z</t>
+    <t>2026-06-20T06:19:43.693Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:45.092Z</t>
   </si>
   <si>
     <t>TC-062</t>
@@ -1024,10 +1021,10 @@
     <t>Verify at least one event card is displayed in the events list.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:43.949Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:45.469Z</t>
+    <t>2026-06-20T06:19:43.737Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:44.221Z</t>
   </si>
   <si>
     <t>TC-063</t>
@@ -1039,10 +1036,10 @@
     <t>Verify event card titles (e.g. "Food Drive") are visible.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:43.979Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:44.614Z</t>
+    <t>2026-06-20T06:19:43.769Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:44.739Z</t>
   </si>
   <si>
     <t>TC-064</t>
@@ -1054,10 +1051,10 @@
     <t>Verify event date labels are formatted and displayed per card.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:44.019Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:44.984Z</t>
+    <t>2026-06-20T06:19:43.800Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:44.913Z</t>
   </si>
   <si>
     <t>TC-065</t>
@@ -1069,10 +1066,7 @@
     <t>Verify location text is shown on each event card.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:44.061Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:45.729Z</t>
+    <t>2026-06-20T06:19:45.039Z</t>
   </si>
   <si>
     <t>TC-066</t>
@@ -1084,10 +1078,10 @@
     <t>Verify volunteer capacity progress bar renders on event cards.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:44.102Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:45.658Z</t>
+    <t>2026-06-20T06:19:43.862Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:45.326Z</t>
   </si>
   <si>
     <t>TC-067</t>
@@ -1099,10 +1093,10 @@
     <t>Verify category classification badge is shown per event.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:44.144Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:45.614Z</t>
+    <t>2026-06-20T06:19:43.893Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:44.912Z</t>
   </si>
   <si>
     <t>TC-068</t>
@@ -1114,10 +1108,10 @@
     <t>Type "Food" in events search and verify matching cards appear.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:44.180Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:44.656Z</t>
+    <t>2026-06-20T06:19:43.925Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:44.796Z</t>
   </si>
   <si>
     <t>TC-069</t>
@@ -1129,10 +1123,10 @@
     <t>Click an event card and verify the event detail sheet expands.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:44.226Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:44.968Z</t>
+    <t>2026-06-20T06:19:43.956Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:44.738Z</t>
   </si>
   <si>
     <t>TC-070</t>
@@ -1144,10 +1138,10 @@
     <t>Verify the event agenda/description paragraph is visible in sheet.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:44.258Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:44.747Z</t>
+    <t>2026-06-20T06:19:43.988Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:44.911Z</t>
   </si>
   <si>
     <t>TC-071</t>
@@ -1159,10 +1153,10 @@
     <t>Verify the list of assigned volunteers appears in event detail.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:44.300Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:44.652Z</t>
+    <t>2026-06-20T06:19:44.019Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:44.741Z</t>
   </si>
   <si>
     <t>TC-072</t>
@@ -1174,10 +1168,10 @@
     <t>Verify clicking close dismisses the event detail sheet.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:44.341Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:45.696Z</t>
+    <t>2026-06-20T06:19:44.050Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:44.751Z</t>
   </si>
   <si>
     <t>TC-073</t>
@@ -1192,10 +1186,10 @@
     <t>Click "Attendance" sidebar item and verify /attendance route loads.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:44.385Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:44.886Z</t>
+    <t>2026-06-20T06:19:44.081Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:45.729Z</t>
   </si>
   <si>
     <t>TC-074</t>
@@ -1207,10 +1201,7 @@
     <t>Verify checked-in count statistics are shown in a metrics bar.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:44.423Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:45.597Z</t>
+    <t>2026-06-20T06:19:45.785Z</t>
   </si>
   <si>
     <t>TC-075</t>
@@ -1222,10 +1213,10 @@
     <t>Verify the attendance log table is rendered with row records.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:44.459Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:45.281Z</t>
+    <t>2026-06-20T06:19:44.159Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:45.025Z</t>
   </si>
   <si>
     <t>TC-076</t>
@@ -1237,10 +1228,10 @@
     <t>Verify table columns (Volunteer, Event, Date, Duration) are labeled.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:44.494Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:45.090Z</t>
+    <t>2026-06-20T06:19:44.190Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:44.784Z</t>
   </si>
   <si>
     <t>TC-077</t>
@@ -1252,10 +1243,7 @@
     <t>Type a volunteer name in search and verify matching log rows.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:44.525Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:45.510Z</t>
+    <t>2026-06-20T06:19:45.936Z</t>
   </si>
   <si>
     <t>TC-078</t>
@@ -1267,10 +1255,10 @@
     <t>Filter attendance records by selecting a specific event.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:44.568Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:44.965Z</t>
+    <t>2026-06-20T06:19:44.252Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:45.873Z</t>
   </si>
   <si>
     <t>TC-079</t>
@@ -1282,10 +1270,10 @@
     <t>Verify the "Check-In" action button is present and clickable.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:44.603Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:45.072Z</t>
+    <t>2026-06-20T06:19:44.283Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:45.598Z</t>
   </si>
   <si>
     <t>TC-080</t>
@@ -1297,10 +1285,10 @@
     <t>Click Check-In and verify the volunteer selection dialog opens.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:44.634Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:45.047Z</t>
+    <t>2026-06-20T06:19:44.315Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:44.866Z</t>
   </si>
   <si>
     <t>TC-081</t>
@@ -1312,10 +1300,10 @@
     <t>Select event and volunteer in dialog, submit and verify toast confirmation.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:44.667Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:46.268Z</t>
+    <t>2026-06-20T06:19:44.346Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:44.726Z</t>
   </si>
   <si>
     <t>TC-082</t>
@@ -1327,10 +1315,10 @@
     <t>Click Export and verify download is triggered for the data.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:44.709Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:45.656Z</t>
+    <t>2026-06-20T06:19:44.378Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:45.129Z</t>
   </si>
   <si>
     <t>TC-083</t>
@@ -1345,10 +1333,10 @@
     <t>Click "Reports" sidebar item and verify /reports route loads.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:44.744Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:45.309Z</t>
+    <t>2026-06-20T06:19:44.423Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:45.817Z</t>
   </si>
   <si>
     <t>TC-084</t>
@@ -1360,10 +1348,10 @@
     <t>Verify multiple charts and analytics sections render on reports page.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:44.776Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:46.220Z</t>
+    <t>2026-06-20T06:19:44.455Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:45.176Z</t>
   </si>
   <si>
     <t>TC-085</t>
@@ -1375,10 +1363,10 @@
     <t>Verify a sortable top contributors table is present on reports screen.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:44.822Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:45.646Z</t>
+    <t>2026-06-20T06:19:44.487Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:45.565Z</t>
   </si>
   <si>
     <t>TC-086</t>
@@ -1390,10 +1378,10 @@
     <t>Verify a date filter/range picker is available on the reports screen.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:44.855Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:45.211Z</t>
+    <t>2026-06-20T06:19:44.518Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:45.703Z</t>
   </si>
   <si>
     <t>TC-087</t>
@@ -1408,10 +1396,10 @@
     <t>Click "AI Assistant" sidebar item and verify /ai-chat route loads.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:44.901Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:46.449Z</t>
+    <t>2026-06-20T06:19:44.548Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:45.639Z</t>
   </si>
   <si>
     <t>TC-088</t>
@@ -1423,10 +1411,10 @@
     <t>Verify "Volt" AI assistant header and intro message is displayed.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:44.942Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:45.810Z</t>
+    <t>2026-06-20T06:19:44.580Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:45.590Z</t>
   </si>
   <si>
     <t>TC-089</t>
@@ -1438,10 +1426,10 @@
     <t>Verify quick-prompt suggestion cards are rendered in the chat view.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:44.985Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:45.464Z</t>
+    <t>2026-06-20T06:19:44.625Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:45.734Z</t>
   </si>
   <si>
     <t>TC-090</t>
@@ -1453,10 +1441,10 @@
     <t>Verify the message input field is visible and accepts typed text.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:45.026Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:46.202Z</t>
+    <t>2026-06-20T06:19:44.657Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:45.271Z</t>
   </si>
   <si>
     <t>TC-091</t>
@@ -1468,10 +1456,10 @@
     <t>Type "Show upcoming events" and press Enter; verify message bubble appears.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:45.069Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:46.101Z</t>
+    <t>2026-06-20T06:19:44.688Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:45.615Z</t>
   </si>
   <si>
     <t>TC-092</t>
@@ -1483,10 +1471,10 @@
     <t>Verify Volt AI returns a response bubble with structured text.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:45.109Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:45.857Z</t>
+    <t>2026-06-20T06:19:44.721Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:45.957Z</t>
   </si>
   <si>
     <t>TC-093</t>
@@ -1498,10 +1486,10 @@
     <t>Type "Generate attendance report" and verify AI processes the request.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:45.151Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:46.739Z</t>
+    <t>2026-06-20T06:19:44.752Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:46.034Z</t>
   </si>
   <si>
     <t>TC-094</t>
@@ -1513,10 +1501,10 @@
     <t>Verify a typing animation/indicator appears while Volt computes reply.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:45.195Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:46.552Z</t>
+    <t>2026-06-20T06:19:44.783Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:45.838Z</t>
   </si>
   <si>
     <t>TC-095</t>
@@ -1531,10 +1519,10 @@
     <t>Click "Settings" sidebar item and verify /settings route loads.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:45.234Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:45.606Z</t>
+    <t>2026-06-20T06:19:44.814Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:45.551Z</t>
   </si>
   <si>
     <t>TC-096</t>
@@ -1546,10 +1534,10 @@
     <t>Verify user name, email, and role appear in the profile section.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:45.271Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:46.767Z</t>
+    <t>2026-06-20T06:19:44.845Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:45.563Z</t>
   </si>
   <si>
     <t>TC-097</t>
@@ -1561,10 +1549,7 @@
     <t>Verify Email/Push notification toggle switches are rendered.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:45.306Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:46.597Z</t>
+    <t>2026-06-20T06:19:45.391Z</t>
   </si>
   <si>
     <t>TC-098</t>
@@ -1576,10 +1561,10 @@
     <t>Click email notification switch and verify it changes state.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:45.340Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:46.998Z</t>
+    <t>2026-06-20T06:19:44.907Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:45.473Z</t>
   </si>
   <si>
     <t>TC-099</t>
@@ -1591,10 +1576,10 @@
     <t>Verify language selection dropdown is present and operable.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:45.370Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:46.774Z</t>
+    <t>2026-06-20T06:19:44.938Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:46.533Z</t>
   </si>
   <si>
     <t>TC-100</t>
@@ -1606,10 +1591,10 @@
     <t>Click "Sign Out" and verify browser is redirected back to /login.</t>
   </si>
   <si>
-    <t>2026-06-14T11:40:45.407Z</t>
-  </si>
-  <si>
-    <t>2026-06-14T11:40:46.760Z</t>
+    <t>2026-06-20T06:19:44.969Z</t>
+  </si>
+  <si>
+    <t>2026-06-20T06:19:46.218Z</t>
   </si>
 </sst>
 </file>
@@ -2375,7 +2360,7 @@
         <v>27</v>
       </c>
       <c r="H9" s="20">
-        <v>1661</v>
+        <v>676</v>
       </c>
       <c r="I9" s="18" t="s">
         <v>28</v>
@@ -2404,7 +2389,7 @@
         <v>33</v>
       </c>
       <c r="H10" s="23">
-        <v>1730</v>
+        <v>1541</v>
       </c>
       <c r="I10" s="22" t="s">
         <v>28</v>
@@ -2433,7 +2418,7 @@
         <v>38</v>
       </c>
       <c r="H11" s="20">
-        <v>735</v>
+        <v>842</v>
       </c>
       <c r="I11" s="18" t="s">
         <v>28</v>
@@ -2462,7 +2447,7 @@
         <v>43</v>
       </c>
       <c r="H12" s="23">
-        <v>1640</v>
+        <v>1020</v>
       </c>
       <c r="I12" s="22" t="s">
         <v>28</v>
@@ -2491,7 +2476,7 @@
         <v>48</v>
       </c>
       <c r="H13" s="20">
-        <v>438</v>
+        <v>1032</v>
       </c>
       <c r="I13" s="18" t="s">
         <v>28</v>
@@ -2520,7 +2505,7 @@
         <v>53</v>
       </c>
       <c r="H14" s="23">
-        <v>656</v>
+        <v>867</v>
       </c>
       <c r="I14" s="22" t="s">
         <v>28</v>
@@ -2549,7 +2534,7 @@
         <v>58</v>
       </c>
       <c r="H15" s="20">
-        <v>1239</v>
+        <v>387</v>
       </c>
       <c r="I15" s="18" t="s">
         <v>28</v>
@@ -2578,7 +2563,7 @@
         <v>63</v>
       </c>
       <c r="H16" s="23">
-        <v>756</v>
+        <v>1355</v>
       </c>
       <c r="I16" s="22" t="s">
         <v>28</v>
@@ -2607,7 +2592,7 @@
         <v>68</v>
       </c>
       <c r="H17" s="20">
-        <v>760</v>
+        <v>1038</v>
       </c>
       <c r="I17" s="18" t="s">
         <v>28</v>
@@ -2636,7 +2621,7 @@
         <v>73</v>
       </c>
       <c r="H18" s="23">
-        <v>1425</v>
+        <v>1391</v>
       </c>
       <c r="I18" s="22" t="s">
         <v>28</v>
@@ -2665,7 +2650,7 @@
         <v>79</v>
       </c>
       <c r="H19" s="20">
-        <v>999</v>
+        <v>1699</v>
       </c>
       <c r="I19" s="18" t="s">
         <v>28</v>
@@ -2694,7 +2679,7 @@
         <v>84</v>
       </c>
       <c r="H20" s="23">
-        <v>1330</v>
+        <v>677</v>
       </c>
       <c r="I20" s="22" t="s">
         <v>28</v>
@@ -2723,7 +2708,7 @@
         <v>89</v>
       </c>
       <c r="H21" s="20">
-        <v>1250</v>
+        <v>956</v>
       </c>
       <c r="I21" s="18" t="s">
         <v>28</v>
@@ -2752,7 +2737,7 @@
         <v>94</v>
       </c>
       <c r="H22" s="23">
-        <v>623</v>
+        <v>530</v>
       </c>
       <c r="I22" s="22" t="s">
         <v>28</v>
@@ -2781,7 +2766,7 @@
         <v>99</v>
       </c>
       <c r="H23" s="20">
-        <v>667</v>
+        <v>520</v>
       </c>
       <c r="I23" s="18" t="s">
         <v>28</v>
@@ -2810,7 +2795,7 @@
         <v>104</v>
       </c>
       <c r="H24" s="23">
-        <v>366</v>
+        <v>587</v>
       </c>
       <c r="I24" s="22" t="s">
         <v>28</v>
@@ -2839,7 +2824,7 @@
         <v>109</v>
       </c>
       <c r="H25" s="20">
-        <v>1548</v>
+        <v>646</v>
       </c>
       <c r="I25" s="18" t="s">
         <v>28</v>
@@ -2868,7 +2853,7 @@
         <v>114</v>
       </c>
       <c r="H26" s="23">
-        <v>1418</v>
+        <v>823</v>
       </c>
       <c r="I26" s="22" t="s">
         <v>28</v>
@@ -2897,7 +2882,7 @@
         <v>119</v>
       </c>
       <c r="H27" s="20">
-        <v>988</v>
+        <v>817</v>
       </c>
       <c r="I27" s="18" t="s">
         <v>28</v>
@@ -2926,7 +2911,7 @@
         <v>124</v>
       </c>
       <c r="H28" s="23">
-        <v>1522</v>
+        <v>879</v>
       </c>
       <c r="I28" s="22" t="s">
         <v>28</v>
@@ -2955,7 +2940,7 @@
         <v>129</v>
       </c>
       <c r="H29" s="20">
-        <v>1211</v>
+        <v>1045</v>
       </c>
       <c r="I29" s="18" t="s">
         <v>28</v>
@@ -2984,7 +2969,7 @@
         <v>134</v>
       </c>
       <c r="H30" s="23">
-        <v>1035</v>
+        <v>931</v>
       </c>
       <c r="I30" s="22" t="s">
         <v>28</v>
@@ -3013,7 +2998,7 @@
         <v>139</v>
       </c>
       <c r="H31" s="20">
-        <v>1159</v>
+        <v>558</v>
       </c>
       <c r="I31" s="18" t="s">
         <v>28</v>
@@ -3042,7 +3027,7 @@
         <v>144</v>
       </c>
       <c r="H32" s="23">
-        <v>825</v>
+        <v>1478</v>
       </c>
       <c r="I32" s="22" t="s">
         <v>28</v>
@@ -3071,7 +3056,7 @@
         <v>150</v>
       </c>
       <c r="H33" s="20">
-        <v>1218</v>
+        <v>1159</v>
       </c>
       <c r="I33" s="18" t="s">
         <v>28</v>
@@ -3100,7 +3085,7 @@
         <v>155</v>
       </c>
       <c r="H34" s="23">
-        <v>1705</v>
+        <v>587</v>
       </c>
       <c r="I34" s="22" t="s">
         <v>28</v>
@@ -3129,7 +3114,7 @@
         <v>160</v>
       </c>
       <c r="H35" s="20">
-        <v>1561</v>
+        <v>498</v>
       </c>
       <c r="I35" s="18" t="s">
         <v>28</v>
@@ -3158,7 +3143,7 @@
         <v>165</v>
       </c>
       <c r="H36" s="23">
-        <v>527</v>
+        <v>1005</v>
       </c>
       <c r="I36" s="22" t="s">
         <v>28</v>
@@ -3187,7 +3172,7 @@
         <v>171</v>
       </c>
       <c r="H37" s="20">
-        <v>1702</v>
+        <v>1305</v>
       </c>
       <c r="I37" s="18" t="s">
         <v>28</v>
@@ -3216,7 +3201,7 @@
         <v>176</v>
       </c>
       <c r="H38" s="23">
-        <v>1274</v>
+        <v>639</v>
       </c>
       <c r="I38" s="22" t="s">
         <v>28</v>
@@ -3245,7 +3230,7 @@
         <v>182</v>
       </c>
       <c r="H39" s="20">
-        <v>511</v>
+        <v>375</v>
       </c>
       <c r="I39" s="18" t="s">
         <v>28</v>
@@ -3274,7 +3259,7 @@
         <v>187</v>
       </c>
       <c r="H40" s="23">
-        <v>1403</v>
+        <v>632</v>
       </c>
       <c r="I40" s="22" t="s">
         <v>28</v>
@@ -3297,13 +3282,13 @@
         <v>25</v>
       </c>
       <c r="F41" s="18" t="s">
-        <v>99</v>
+        <v>191</v>
       </c>
       <c r="G41" s="18" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="H41" s="20">
-        <v>1404</v>
+        <v>1011</v>
       </c>
       <c r="I41" s="18" t="s">
         <v>28</v>
@@ -3311,28 +3296,28 @@
     </row>
     <row r="42" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="21" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B42" s="22" t="s">
         <v>178</v>
       </c>
       <c r="C42" s="22" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D42" s="22" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E42" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F42" s="22" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G42" s="22" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="H42" s="23">
-        <v>431</v>
+        <v>616</v>
       </c>
       <c r="I42" s="22" t="s">
         <v>28</v>
@@ -3340,28 +3325,28 @@
     </row>
     <row r="43" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="17" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B43" s="18" t="s">
         <v>178</v>
       </c>
       <c r="C43" s="18" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D43" s="18" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="E43" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F43" s="18" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="G43" s="18" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="H43" s="20">
-        <v>1718</v>
+        <v>985</v>
       </c>
       <c r="I43" s="18" t="s">
         <v>28</v>
@@ -3369,28 +3354,28 @@
     </row>
     <row r="44" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="21" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B44" s="22" t="s">
         <v>178</v>
       </c>
       <c r="C44" s="22" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D44" s="22" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E44" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F44" s="22" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="G44" s="22" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="H44" s="23">
-        <v>736</v>
+        <v>1160</v>
       </c>
       <c r="I44" s="22" t="s">
         <v>28</v>
@@ -3398,28 +3383,28 @@
     </row>
     <row r="45" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="17" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B45" s="18" t="s">
         <v>178</v>
       </c>
       <c r="C45" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D45" s="18" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E45" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F45" s="18" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="G45" s="18" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="H45" s="20">
-        <v>393</v>
+        <v>1660</v>
       </c>
       <c r="I45" s="18" t="s">
         <v>28</v>
@@ -3427,28 +3412,28 @@
     </row>
     <row r="46" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="21" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B46" s="22" t="s">
         <v>178</v>
       </c>
       <c r="C46" s="22" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D46" s="22" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="E46" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F46" s="22" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="G46" s="22" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="H46" s="23">
-        <v>407</v>
+        <v>1027</v>
       </c>
       <c r="I46" s="22" t="s">
         <v>28</v>
@@ -3456,28 +3441,28 @@
     </row>
     <row r="47" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="17" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B47" s="18" t="s">
         <v>178</v>
       </c>
       <c r="C47" s="18" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D47" s="18" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E47" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F47" s="18" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="G47" s="18" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="H47" s="20">
-        <v>702</v>
+        <v>1390</v>
       </c>
       <c r="I47" s="18" t="s">
         <v>28</v>
@@ -3485,28 +3470,28 @@
     </row>
     <row r="48" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="21" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B48" s="22" t="s">
         <v>178</v>
       </c>
       <c r="C48" s="22" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D48" s="22" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E48" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F48" s="22" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G48" s="22" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="H48" s="23">
-        <v>1111</v>
+        <v>703</v>
       </c>
       <c r="I48" s="22" t="s">
         <v>28</v>
@@ -3514,28 +3499,28 @@
     </row>
     <row r="49" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" s="17" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B49" s="18" t="s">
         <v>178</v>
       </c>
       <c r="C49" s="18" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D49" s="18" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E49" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F49" s="18" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="G49" s="18" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="H49" s="20">
-        <v>1426</v>
+        <v>760</v>
       </c>
       <c r="I49" s="18" t="s">
         <v>28</v>
@@ -3543,28 +3528,28 @@
     </row>
     <row r="50" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="21" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B50" s="22" t="s">
         <v>178</v>
       </c>
       <c r="C50" s="22" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D50" s="22" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E50" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F50" s="22" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="G50" s="22" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="H50" s="23">
-        <v>1585</v>
+        <v>1404</v>
       </c>
       <c r="I50" s="22" t="s">
         <v>28</v>
@@ -3572,28 +3557,28 @@
     </row>
     <row r="51" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" s="17" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B51" s="18" t="s">
         <v>178</v>
       </c>
       <c r="C51" s="18" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D51" s="18" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E51" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F51" s="18" t="s">
-        <v>240</v>
+        <v>160</v>
       </c>
       <c r="G51" s="18" t="s">
         <v>241</v>
       </c>
       <c r="H51" s="20">
-        <v>498</v>
+        <v>885</v>
       </c>
       <c r="I51" s="18" t="s">
         <v>28</v>
@@ -3622,7 +3607,7 @@
         <v>246</v>
       </c>
       <c r="H52" s="23">
-        <v>381</v>
+        <v>717</v>
       </c>
       <c r="I52" s="22" t="s">
         <v>28</v>
@@ -3651,7 +3636,7 @@
         <v>251</v>
       </c>
       <c r="H53" s="20">
-        <v>743</v>
+        <v>589</v>
       </c>
       <c r="I53" s="18" t="s">
         <v>28</v>
@@ -3680,7 +3665,7 @@
         <v>257</v>
       </c>
       <c r="H54" s="23">
-        <v>1121</v>
+        <v>1602</v>
       </c>
       <c r="I54" s="22" t="s">
         <v>28</v>
@@ -3709,7 +3694,7 @@
         <v>262</v>
       </c>
       <c r="H55" s="20">
-        <v>660</v>
+        <v>407</v>
       </c>
       <c r="I55" s="18" t="s">
         <v>28</v>
@@ -3738,7 +3723,7 @@
         <v>267</v>
       </c>
       <c r="H56" s="23">
-        <v>1481</v>
+        <v>955</v>
       </c>
       <c r="I56" s="22" t="s">
         <v>28</v>
@@ -3767,7 +3752,7 @@
         <v>272</v>
       </c>
       <c r="H57" s="20">
-        <v>1067</v>
+        <v>916</v>
       </c>
       <c r="I57" s="18" t="s">
         <v>28</v>
@@ -3796,7 +3781,7 @@
         <v>277</v>
       </c>
       <c r="H58" s="23">
-        <v>1244</v>
+        <v>1346</v>
       </c>
       <c r="I58" s="22" t="s">
         <v>28</v>
@@ -3825,7 +3810,7 @@
         <v>282</v>
       </c>
       <c r="H59" s="20">
-        <v>852</v>
+        <v>748</v>
       </c>
       <c r="I59" s="18" t="s">
         <v>28</v>
@@ -3854,7 +3839,7 @@
         <v>287</v>
       </c>
       <c r="H60" s="23">
-        <v>478</v>
+        <v>1552</v>
       </c>
       <c r="I60" s="22" t="s">
         <v>28</v>
@@ -3883,7 +3868,7 @@
         <v>292</v>
       </c>
       <c r="H61" s="20">
-        <v>898</v>
+        <v>1435</v>
       </c>
       <c r="I61" s="18" t="s">
         <v>28</v>
@@ -3912,7 +3897,7 @@
         <v>297</v>
       </c>
       <c r="H62" s="23">
-        <v>834</v>
+        <v>1247</v>
       </c>
       <c r="I62" s="22" t="s">
         <v>28</v>
@@ -3941,7 +3926,7 @@
         <v>302</v>
       </c>
       <c r="H63" s="20">
-        <v>1593</v>
+        <v>1738</v>
       </c>
       <c r="I63" s="18" t="s">
         <v>28</v>
@@ -3970,7 +3955,7 @@
         <v>307</v>
       </c>
       <c r="H64" s="23">
-        <v>1679</v>
+        <v>511</v>
       </c>
       <c r="I64" s="22" t="s">
         <v>28</v>
@@ -3999,7 +3984,7 @@
         <v>312</v>
       </c>
       <c r="H65" s="20">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="I65" s="18" t="s">
         <v>28</v>
@@ -4028,7 +4013,7 @@
         <v>317</v>
       </c>
       <c r="H66" s="23">
-        <v>1115</v>
+        <v>500</v>
       </c>
       <c r="I66" s="22" t="s">
         <v>28</v>
@@ -4057,7 +4042,7 @@
         <v>322</v>
       </c>
       <c r="H67" s="20">
-        <v>988</v>
+        <v>851</v>
       </c>
       <c r="I67" s="18" t="s">
         <v>28</v>
@@ -4080,13 +4065,13 @@
         <v>25</v>
       </c>
       <c r="F68" s="22" t="s">
+        <v>262</v>
+      </c>
+      <c r="G68" s="22" t="s">
         <v>326</v>
       </c>
-      <c r="G68" s="22" t="s">
-        <v>327</v>
-      </c>
       <c r="H68" s="23">
-        <v>1499</v>
+        <v>791</v>
       </c>
       <c r="I68" s="22" t="s">
         <v>28</v>
@@ -4094,28 +4079,28 @@
     </row>
     <row r="69" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" s="17" t="s">
+        <v>327</v>
+      </c>
+      <c r="B69" s="18" t="s">
         <v>328</v>
       </c>
-      <c r="B69" s="18" t="s">
+      <c r="C69" s="18" t="s">
         <v>329</v>
       </c>
-      <c r="C69" s="18" t="s">
+      <c r="D69" s="18" t="s">
         <v>330</v>
       </c>
-      <c r="D69" s="18" t="s">
+      <c r="E69" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F69" s="18" t="s">
         <v>331</v>
       </c>
-      <c r="E69" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F69" s="18" t="s">
+      <c r="G69" s="18" t="s">
         <v>332</v>
       </c>
-      <c r="G69" s="18" t="s">
-        <v>333</v>
-      </c>
       <c r="H69" s="20">
-        <v>1591</v>
+        <v>1399</v>
       </c>
       <c r="I69" s="18" t="s">
         <v>28</v>
@@ -4123,28 +4108,28 @@
     </row>
     <row r="70" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" s="21" t="s">
+        <v>333</v>
+      </c>
+      <c r="B70" s="22" t="s">
+        <v>328</v>
+      </c>
+      <c r="C70" s="22" t="s">
         <v>334</v>
       </c>
-      <c r="B70" s="22" t="s">
-        <v>329</v>
-      </c>
-      <c r="C70" s="22" t="s">
+      <c r="D70" s="22" t="s">
         <v>335</v>
       </c>
-      <c r="D70" s="22" t="s">
+      <c r="E70" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F70" s="22" t="s">
         <v>336</v>
       </c>
-      <c r="E70" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F70" s="22" t="s">
+      <c r="G70" s="22" t="s">
         <v>337</v>
       </c>
-      <c r="G70" s="22" t="s">
-        <v>338</v>
-      </c>
       <c r="H70" s="23">
-        <v>1520</v>
+        <v>484</v>
       </c>
       <c r="I70" s="22" t="s">
         <v>28</v>
@@ -4152,28 +4137,28 @@
     </row>
     <row r="71" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" s="17" t="s">
+        <v>338</v>
+      </c>
+      <c r="B71" s="18" t="s">
+        <v>328</v>
+      </c>
+      <c r="C71" s="18" t="s">
         <v>339</v>
       </c>
-      <c r="B71" s="18" t="s">
-        <v>329</v>
-      </c>
-      <c r="C71" s="18" t="s">
+      <c r="D71" s="18" t="s">
         <v>340</v>
       </c>
-      <c r="D71" s="18" t="s">
+      <c r="E71" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F71" s="18" t="s">
         <v>341</v>
       </c>
-      <c r="E71" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F71" s="18" t="s">
+      <c r="G71" s="18" t="s">
         <v>342</v>
       </c>
-      <c r="G71" s="18" t="s">
-        <v>343</v>
-      </c>
       <c r="H71" s="20">
-        <v>635</v>
+        <v>970</v>
       </c>
       <c r="I71" s="18" t="s">
         <v>28</v>
@@ -4181,28 +4166,28 @@
     </row>
     <row r="72" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" s="21" t="s">
+        <v>343</v>
+      </c>
+      <c r="B72" s="22" t="s">
+        <v>328</v>
+      </c>
+      <c r="C72" s="22" t="s">
         <v>344</v>
       </c>
-      <c r="B72" s="22" t="s">
-        <v>329</v>
-      </c>
-      <c r="C72" s="22" t="s">
+      <c r="D72" s="22" t="s">
         <v>345</v>
       </c>
-      <c r="D72" s="22" t="s">
+      <c r="E72" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F72" s="22" t="s">
         <v>346</v>
       </c>
-      <c r="E72" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F72" s="22" t="s">
+      <c r="G72" s="22" t="s">
         <v>347</v>
       </c>
-      <c r="G72" s="22" t="s">
-        <v>348</v>
-      </c>
       <c r="H72" s="23">
-        <v>965</v>
+        <v>1113</v>
       </c>
       <c r="I72" s="22" t="s">
         <v>28</v>
@@ -4210,28 +4195,28 @@
     </row>
     <row r="73" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" s="17" t="s">
+        <v>348</v>
+      </c>
+      <c r="B73" s="18" t="s">
+        <v>328</v>
+      </c>
+      <c r="C73" s="18" t="s">
         <v>349</v>
       </c>
-      <c r="B73" s="18" t="s">
-        <v>329</v>
-      </c>
-      <c r="C73" s="18" t="s">
+      <c r="D73" s="18" t="s">
         <v>350</v>
       </c>
-      <c r="D73" s="18" t="s">
+      <c r="E73" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F73" s="18" t="s">
+        <v>192</v>
+      </c>
+      <c r="G73" s="18" t="s">
         <v>351</v>
       </c>
-      <c r="E73" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F73" s="18" t="s">
-        <v>352</v>
-      </c>
-      <c r="G73" s="18" t="s">
-        <v>353</v>
-      </c>
       <c r="H73" s="20">
-        <v>1668</v>
+        <v>1208</v>
       </c>
       <c r="I73" s="18" t="s">
         <v>28</v>
@@ -4239,28 +4224,28 @@
     </row>
     <row r="74" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" s="21" t="s">
+        <v>352</v>
+      </c>
+      <c r="B74" s="22" t="s">
+        <v>328</v>
+      </c>
+      <c r="C74" s="22" t="s">
+        <v>353</v>
+      </c>
+      <c r="D74" s="22" t="s">
         <v>354</v>
       </c>
-      <c r="B74" s="22" t="s">
-        <v>329</v>
-      </c>
-      <c r="C74" s="22" t="s">
+      <c r="E74" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F74" s="22" t="s">
         <v>355</v>
       </c>
-      <c r="D74" s="22" t="s">
+      <c r="G74" s="22" t="s">
         <v>356</v>
       </c>
-      <c r="E74" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F74" s="22" t="s">
-        <v>357</v>
-      </c>
-      <c r="G74" s="22" t="s">
-        <v>358</v>
-      </c>
       <c r="H74" s="23">
-        <v>1556</v>
+        <v>1464</v>
       </c>
       <c r="I74" s="22" t="s">
         <v>28</v>
@@ -4268,28 +4253,28 @@
     </row>
     <row r="75" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75" s="17" t="s">
+        <v>357</v>
+      </c>
+      <c r="B75" s="18" t="s">
+        <v>328</v>
+      </c>
+      <c r="C75" s="18" t="s">
+        <v>358</v>
+      </c>
+      <c r="D75" s="18" t="s">
         <v>359</v>
       </c>
-      <c r="B75" s="18" t="s">
-        <v>329</v>
-      </c>
-      <c r="C75" s="18" t="s">
+      <c r="E75" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F75" s="18" t="s">
         <v>360</v>
       </c>
-      <c r="D75" s="18" t="s">
+      <c r="G75" s="18" t="s">
         <v>361</v>
       </c>
-      <c r="E75" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F75" s="18" t="s">
-        <v>362</v>
-      </c>
-      <c r="G75" s="18" t="s">
-        <v>363</v>
-      </c>
       <c r="H75" s="20">
-        <v>1470</v>
+        <v>1019</v>
       </c>
       <c r="I75" s="18" t="s">
         <v>28</v>
@@ -4297,28 +4282,28 @@
     </row>
     <row r="76" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76" s="21" t="s">
+        <v>362</v>
+      </c>
+      <c r="B76" s="22" t="s">
+        <v>328</v>
+      </c>
+      <c r="C76" s="22" t="s">
+        <v>363</v>
+      </c>
+      <c r="D76" s="22" t="s">
         <v>364</v>
       </c>
-      <c r="B76" s="22" t="s">
-        <v>329</v>
-      </c>
-      <c r="C76" s="22" t="s">
+      <c r="E76" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F76" s="22" t="s">
         <v>365</v>
       </c>
-      <c r="D76" s="22" t="s">
+      <c r="G76" s="22" t="s">
         <v>366</v>
       </c>
-      <c r="E76" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F76" s="22" t="s">
-        <v>367</v>
-      </c>
-      <c r="G76" s="22" t="s">
-        <v>368</v>
-      </c>
       <c r="H76" s="23">
-        <v>476</v>
+        <v>871</v>
       </c>
       <c r="I76" s="22" t="s">
         <v>28</v>
@@ -4326,28 +4311,28 @@
     </row>
     <row r="77" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77" s="17" t="s">
+        <v>367</v>
+      </c>
+      <c r="B77" s="18" t="s">
+        <v>328</v>
+      </c>
+      <c r="C77" s="18" t="s">
+        <v>368</v>
+      </c>
+      <c r="D77" s="18" t="s">
         <v>369</v>
       </c>
-      <c r="B77" s="18" t="s">
-        <v>329</v>
-      </c>
-      <c r="C77" s="18" t="s">
+      <c r="E77" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F77" s="18" t="s">
         <v>370</v>
       </c>
-      <c r="D77" s="18" t="s">
+      <c r="G77" s="18" t="s">
         <v>371</v>
       </c>
-      <c r="E77" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F77" s="18" t="s">
-        <v>372</v>
-      </c>
-      <c r="G77" s="18" t="s">
-        <v>373</v>
-      </c>
       <c r="H77" s="20">
-        <v>742</v>
+        <v>782</v>
       </c>
       <c r="I77" s="18" t="s">
         <v>28</v>
@@ -4355,28 +4340,28 @@
     </row>
     <row r="78" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78" s="21" t="s">
+        <v>372</v>
+      </c>
+      <c r="B78" s="22" t="s">
+        <v>328</v>
+      </c>
+      <c r="C78" s="22" t="s">
+        <v>373</v>
+      </c>
+      <c r="D78" s="22" t="s">
         <v>374</v>
       </c>
-      <c r="B78" s="22" t="s">
-        <v>329</v>
-      </c>
-      <c r="C78" s="22" t="s">
+      <c r="E78" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F78" s="22" t="s">
         <v>375</v>
       </c>
-      <c r="D78" s="22" t="s">
+      <c r="G78" s="22" t="s">
         <v>376</v>
       </c>
-      <c r="E78" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F78" s="22" t="s">
-        <v>377</v>
-      </c>
-      <c r="G78" s="22" t="s">
-        <v>378</v>
-      </c>
       <c r="H78" s="23">
-        <v>489</v>
+        <v>923</v>
       </c>
       <c r="I78" s="22" t="s">
         <v>28</v>
@@ -4384,28 +4369,28 @@
     </row>
     <row r="79" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79" s="17" t="s">
+        <v>377</v>
+      </c>
+      <c r="B79" s="18" t="s">
+        <v>328</v>
+      </c>
+      <c r="C79" s="18" t="s">
+        <v>378</v>
+      </c>
+      <c r="D79" s="18" t="s">
         <v>379</v>
       </c>
-      <c r="B79" s="18" t="s">
-        <v>329</v>
-      </c>
-      <c r="C79" s="18" t="s">
+      <c r="E79" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F79" s="18" t="s">
         <v>380</v>
       </c>
-      <c r="D79" s="18" t="s">
+      <c r="G79" s="18" t="s">
         <v>381</v>
       </c>
-      <c r="E79" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F79" s="18" t="s">
-        <v>382</v>
-      </c>
-      <c r="G79" s="18" t="s">
-        <v>383</v>
-      </c>
       <c r="H79" s="20">
-        <v>352</v>
+        <v>722</v>
       </c>
       <c r="I79" s="18" t="s">
         <v>28</v>
@@ -4413,28 +4398,28 @@
     </row>
     <row r="80" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80" s="21" t="s">
+        <v>382</v>
+      </c>
+      <c r="B80" s="22" t="s">
+        <v>328</v>
+      </c>
+      <c r="C80" s="22" t="s">
+        <v>383</v>
+      </c>
+      <c r="D80" s="22" t="s">
         <v>384</v>
       </c>
-      <c r="B80" s="22" t="s">
-        <v>329</v>
-      </c>
-      <c r="C80" s="22" t="s">
+      <c r="E80" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F80" s="22" t="s">
         <v>385</v>
       </c>
-      <c r="D80" s="22" t="s">
+      <c r="G80" s="22" t="s">
         <v>386</v>
       </c>
-      <c r="E80" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F80" s="22" t="s">
-        <v>387</v>
-      </c>
-      <c r="G80" s="22" t="s">
-        <v>388</v>
-      </c>
       <c r="H80" s="23">
-        <v>1355</v>
+        <v>701</v>
       </c>
       <c r="I80" s="22" t="s">
         <v>28</v>
@@ -4442,28 +4427,28 @@
     </row>
     <row r="81" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A81" s="17" t="s">
+        <v>387</v>
+      </c>
+      <c r="B81" s="18" t="s">
+        <v>388</v>
+      </c>
+      <c r="C81" s="18" t="s">
         <v>389</v>
       </c>
-      <c r="B81" s="18" t="s">
+      <c r="D81" s="18" t="s">
         <v>390</v>
       </c>
-      <c r="C81" s="18" t="s">
+      <c r="E81" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F81" s="18" t="s">
         <v>391</v>
       </c>
-      <c r="D81" s="18" t="s">
+      <c r="G81" s="18" t="s">
         <v>392</v>
       </c>
-      <c r="E81" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F81" s="18" t="s">
-        <v>393</v>
-      </c>
-      <c r="G81" s="18" t="s">
-        <v>394</v>
-      </c>
       <c r="H81" s="20">
-        <v>501</v>
+        <v>1648</v>
       </c>
       <c r="I81" s="18" t="s">
         <v>28</v>
@@ -4471,28 +4456,28 @@
     </row>
     <row r="82" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82" s="21" t="s">
+        <v>393</v>
+      </c>
+      <c r="B82" s="22" t="s">
+        <v>388</v>
+      </c>
+      <c r="C82" s="22" t="s">
+        <v>394</v>
+      </c>
+      <c r="D82" s="22" t="s">
         <v>395</v>
       </c>
-      <c r="B82" s="22" t="s">
-        <v>390</v>
-      </c>
-      <c r="C82" s="22" t="s">
+      <c r="E82" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F82" s="22" t="s">
+        <v>282</v>
+      </c>
+      <c r="G82" s="22" t="s">
         <v>396</v>
       </c>
-      <c r="D82" s="22" t="s">
-        <v>397</v>
-      </c>
-      <c r="E82" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F82" s="22" t="s">
-        <v>398</v>
-      </c>
-      <c r="G82" s="22" t="s">
-        <v>399</v>
-      </c>
       <c r="H82" s="23">
-        <v>1174</v>
+        <v>1658</v>
       </c>
       <c r="I82" s="22" t="s">
         <v>28</v>
@@ -4500,28 +4485,28 @@
     </row>
     <row r="83" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" s="17" t="s">
+        <v>397</v>
+      </c>
+      <c r="B83" s="18" t="s">
+        <v>388</v>
+      </c>
+      <c r="C83" s="18" t="s">
+        <v>398</v>
+      </c>
+      <c r="D83" s="18" t="s">
+        <v>399</v>
+      </c>
+      <c r="E83" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F83" s="18" t="s">
         <v>400</v>
       </c>
-      <c r="B83" s="18" t="s">
-        <v>390</v>
-      </c>
-      <c r="C83" s="18" t="s">
+      <c r="G83" s="18" t="s">
         <v>401</v>
       </c>
-      <c r="D83" s="18" t="s">
-        <v>402</v>
-      </c>
-      <c r="E83" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F83" s="18" t="s">
-        <v>403</v>
-      </c>
-      <c r="G83" s="18" t="s">
-        <v>404</v>
-      </c>
       <c r="H83" s="20">
-        <v>822</v>
+        <v>866</v>
       </c>
       <c r="I83" s="18" t="s">
         <v>28</v>
@@ -4529,28 +4514,28 @@
     </row>
     <row r="84" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84" s="21" t="s">
+        <v>402</v>
+      </c>
+      <c r="B84" s="22" t="s">
+        <v>388</v>
+      </c>
+      <c r="C84" s="22" t="s">
+        <v>403</v>
+      </c>
+      <c r="D84" s="22" t="s">
+        <v>404</v>
+      </c>
+      <c r="E84" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F84" s="22" t="s">
         <v>405</v>
       </c>
-      <c r="B84" s="22" t="s">
-        <v>390</v>
-      </c>
-      <c r="C84" s="22" t="s">
+      <c r="G84" s="22" t="s">
         <v>406</v>
       </c>
-      <c r="D84" s="22" t="s">
-        <v>407</v>
-      </c>
-      <c r="E84" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F84" s="22" t="s">
-        <v>408</v>
-      </c>
-      <c r="G84" s="22" t="s">
-        <v>409</v>
-      </c>
       <c r="H84" s="23">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="I84" s="22" t="s">
         <v>28</v>
@@ -4558,28 +4543,28 @@
     </row>
     <row r="85" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85" s="17" t="s">
+        <v>407</v>
+      </c>
+      <c r="B85" s="18" t="s">
+        <v>388</v>
+      </c>
+      <c r="C85" s="18" t="s">
+        <v>408</v>
+      </c>
+      <c r="D85" s="18" t="s">
+        <v>409</v>
+      </c>
+      <c r="E85" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F85" s="18" t="s">
+        <v>337</v>
+      </c>
+      <c r="G85" s="18" t="s">
         <v>410</v>
       </c>
-      <c r="B85" s="18" t="s">
-        <v>390</v>
-      </c>
-      <c r="C85" s="18" t="s">
-        <v>411</v>
-      </c>
-      <c r="D85" s="18" t="s">
-        <v>412</v>
-      </c>
-      <c r="E85" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F85" s="18" t="s">
-        <v>413</v>
-      </c>
-      <c r="G85" s="18" t="s">
-        <v>414</v>
-      </c>
       <c r="H85" s="20">
-        <v>985</v>
+        <v>1715</v>
       </c>
       <c r="I85" s="18" t="s">
         <v>28</v>
@@ -4587,28 +4572,28 @@
     </row>
     <row r="86" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86" s="21" t="s">
+        <v>411</v>
+      </c>
+      <c r="B86" s="22" t="s">
+        <v>388</v>
+      </c>
+      <c r="C86" s="22" t="s">
+        <v>412</v>
+      </c>
+      <c r="D86" s="22" t="s">
+        <v>413</v>
+      </c>
+      <c r="E86" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F86" s="22" t="s">
+        <v>414</v>
+      </c>
+      <c r="G86" s="22" t="s">
         <v>415</v>
       </c>
-      <c r="B86" s="22" t="s">
-        <v>390</v>
-      </c>
-      <c r="C86" s="22" t="s">
-        <v>416</v>
-      </c>
-      <c r="D86" s="22" t="s">
-        <v>417</v>
-      </c>
-      <c r="E86" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F86" s="22" t="s">
-        <v>418</v>
-      </c>
-      <c r="G86" s="22" t="s">
-        <v>419</v>
-      </c>
       <c r="H86" s="23">
-        <v>397</v>
+        <v>1621</v>
       </c>
       <c r="I86" s="22" t="s">
         <v>28</v>
@@ -4616,28 +4601,28 @@
     </row>
     <row r="87" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87" s="17" t="s">
+        <v>416</v>
+      </c>
+      <c r="B87" s="18" t="s">
+        <v>388</v>
+      </c>
+      <c r="C87" s="18" t="s">
+        <v>417</v>
+      </c>
+      <c r="D87" s="18" t="s">
+        <v>418</v>
+      </c>
+      <c r="E87" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F87" s="18" t="s">
+        <v>419</v>
+      </c>
+      <c r="G87" s="18" t="s">
         <v>420</v>
       </c>
-      <c r="B87" s="18" t="s">
-        <v>390</v>
-      </c>
-      <c r="C87" s="18" t="s">
-        <v>421</v>
-      </c>
-      <c r="D87" s="18" t="s">
-        <v>422</v>
-      </c>
-      <c r="E87" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F87" s="18" t="s">
-        <v>423</v>
-      </c>
-      <c r="G87" s="18" t="s">
-        <v>424</v>
-      </c>
       <c r="H87" s="20">
-        <v>469</v>
+        <v>1315</v>
       </c>
       <c r="I87" s="18" t="s">
         <v>28</v>
@@ -4645,28 +4630,28 @@
     </row>
     <row r="88" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88" s="21" t="s">
+        <v>421</v>
+      </c>
+      <c r="B88" s="22" t="s">
+        <v>388</v>
+      </c>
+      <c r="C88" s="22" t="s">
+        <v>422</v>
+      </c>
+      <c r="D88" s="22" t="s">
+        <v>423</v>
+      </c>
+      <c r="E88" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F88" s="22" t="s">
+        <v>424</v>
+      </c>
+      <c r="G88" s="22" t="s">
         <v>425</v>
       </c>
-      <c r="B88" s="22" t="s">
-        <v>390</v>
-      </c>
-      <c r="C88" s="22" t="s">
-        <v>426</v>
-      </c>
-      <c r="D88" s="22" t="s">
-        <v>427</v>
-      </c>
-      <c r="E88" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F88" s="22" t="s">
-        <v>428</v>
-      </c>
-      <c r="G88" s="22" t="s">
-        <v>429</v>
-      </c>
       <c r="H88" s="23">
-        <v>413</v>
+        <v>551</v>
       </c>
       <c r="I88" s="22" t="s">
         <v>28</v>
@@ -4674,28 +4659,28 @@
     </row>
     <row r="89" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89" s="17" t="s">
+        <v>426</v>
+      </c>
+      <c r="B89" s="18" t="s">
+        <v>388</v>
+      </c>
+      <c r="C89" s="18" t="s">
+        <v>427</v>
+      </c>
+      <c r="D89" s="18" t="s">
+        <v>428</v>
+      </c>
+      <c r="E89" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F89" s="18" t="s">
+        <v>429</v>
+      </c>
+      <c r="G89" s="18" t="s">
         <v>430</v>
       </c>
-      <c r="B89" s="18" t="s">
-        <v>390</v>
-      </c>
-      <c r="C89" s="18" t="s">
-        <v>431</v>
-      </c>
-      <c r="D89" s="18" t="s">
-        <v>432</v>
-      </c>
-      <c r="E89" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F89" s="18" t="s">
-        <v>433</v>
-      </c>
-      <c r="G89" s="18" t="s">
-        <v>434</v>
-      </c>
       <c r="H89" s="20">
-        <v>1601</v>
+        <v>380</v>
       </c>
       <c r="I89" s="18" t="s">
         <v>28</v>
@@ -4703,28 +4688,28 @@
     </row>
     <row r="90" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90" s="21" t="s">
+        <v>431</v>
+      </c>
+      <c r="B90" s="22" t="s">
+        <v>388</v>
+      </c>
+      <c r="C90" s="22" t="s">
+        <v>432</v>
+      </c>
+      <c r="D90" s="22" t="s">
+        <v>433</v>
+      </c>
+      <c r="E90" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F90" s="22" t="s">
+        <v>434</v>
+      </c>
+      <c r="G90" s="22" t="s">
         <v>435</v>
       </c>
-      <c r="B90" s="22" t="s">
-        <v>390</v>
-      </c>
-      <c r="C90" s="22" t="s">
-        <v>436</v>
-      </c>
-      <c r="D90" s="22" t="s">
-        <v>437</v>
-      </c>
-      <c r="E90" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F90" s="22" t="s">
-        <v>438</v>
-      </c>
-      <c r="G90" s="22" t="s">
-        <v>439</v>
-      </c>
       <c r="H90" s="23">
-        <v>947</v>
+        <v>751</v>
       </c>
       <c r="I90" s="22" t="s">
         <v>28</v>
@@ -4732,28 +4717,28 @@
     </row>
     <row r="91" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91" s="17" t="s">
+        <v>436</v>
+      </c>
+      <c r="B91" s="18" t="s">
+        <v>437</v>
+      </c>
+      <c r="C91" s="18" t="s">
+        <v>438</v>
+      </c>
+      <c r="D91" s="18" t="s">
+        <v>439</v>
+      </c>
+      <c r="E91" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F91" s="18" t="s">
         <v>440</v>
       </c>
-      <c r="B91" s="18" t="s">
+      <c r="G91" s="18" t="s">
         <v>441</v>
       </c>
-      <c r="C91" s="18" t="s">
-        <v>442</v>
-      </c>
-      <c r="D91" s="18" t="s">
-        <v>443</v>
-      </c>
-      <c r="E91" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F91" s="18" t="s">
-        <v>444</v>
-      </c>
-      <c r="G91" s="18" t="s">
-        <v>445</v>
-      </c>
       <c r="H91" s="20">
-        <v>565</v>
+        <v>1394</v>
       </c>
       <c r="I91" s="18" t="s">
         <v>28</v>
@@ -4761,28 +4746,28 @@
     </row>
     <row r="92" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92" s="21" t="s">
+        <v>442</v>
+      </c>
+      <c r="B92" s="22" t="s">
+        <v>437</v>
+      </c>
+      <c r="C92" s="22" t="s">
+        <v>443</v>
+      </c>
+      <c r="D92" s="22" t="s">
+        <v>444</v>
+      </c>
+      <c r="E92" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F92" s="22" t="s">
+        <v>445</v>
+      </c>
+      <c r="G92" s="22" t="s">
         <v>446</v>
       </c>
-      <c r="B92" s="22" t="s">
-        <v>441</v>
-      </c>
-      <c r="C92" s="22" t="s">
-        <v>447</v>
-      </c>
-      <c r="D92" s="22" t="s">
-        <v>448</v>
-      </c>
-      <c r="E92" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F92" s="22" t="s">
-        <v>449</v>
-      </c>
-      <c r="G92" s="22" t="s">
-        <v>450</v>
-      </c>
       <c r="H92" s="23">
-        <v>1444</v>
+        <v>721</v>
       </c>
       <c r="I92" s="22" t="s">
         <v>28</v>
@@ -4790,28 +4775,28 @@
     </row>
     <row r="93" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A93" s="17" t="s">
+        <v>447</v>
+      </c>
+      <c r="B93" s="18" t="s">
+        <v>437</v>
+      </c>
+      <c r="C93" s="18" t="s">
+        <v>448</v>
+      </c>
+      <c r="D93" s="18" t="s">
+        <v>449</v>
+      </c>
+      <c r="E93" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F93" s="18" t="s">
+        <v>450</v>
+      </c>
+      <c r="G93" s="18" t="s">
         <v>451</v>
       </c>
-      <c r="B93" s="18" t="s">
-        <v>441</v>
-      </c>
-      <c r="C93" s="18" t="s">
-        <v>452</v>
-      </c>
-      <c r="D93" s="18" t="s">
-        <v>453</v>
-      </c>
-      <c r="E93" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F93" s="18" t="s">
-        <v>454</v>
-      </c>
-      <c r="G93" s="18" t="s">
-        <v>455</v>
-      </c>
       <c r="H93" s="20">
-        <v>824</v>
+        <v>1078</v>
       </c>
       <c r="I93" s="18" t="s">
         <v>28</v>
@@ -4819,28 +4804,28 @@
     </row>
     <row r="94" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A94" s="21" t="s">
+        <v>452</v>
+      </c>
+      <c r="B94" s="22" t="s">
+        <v>437</v>
+      </c>
+      <c r="C94" s="22" t="s">
+        <v>453</v>
+      </c>
+      <c r="D94" s="22" t="s">
+        <v>454</v>
+      </c>
+      <c r="E94" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F94" s="22" t="s">
+        <v>455</v>
+      </c>
+      <c r="G94" s="22" t="s">
         <v>456</v>
       </c>
-      <c r="B94" s="22" t="s">
-        <v>441</v>
-      </c>
-      <c r="C94" s="22" t="s">
-        <v>457</v>
-      </c>
-      <c r="D94" s="22" t="s">
-        <v>458</v>
-      </c>
-      <c r="E94" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F94" s="22" t="s">
-        <v>459</v>
-      </c>
-      <c r="G94" s="22" t="s">
-        <v>460</v>
-      </c>
       <c r="H94" s="23">
-        <v>356</v>
+        <v>1185</v>
       </c>
       <c r="I94" s="22" t="s">
         <v>28</v>
@@ -4848,28 +4833,28 @@
     </row>
     <row r="95" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A95" s="17" t="s">
+        <v>457</v>
+      </c>
+      <c r="B95" s="18" t="s">
+        <v>458</v>
+      </c>
+      <c r="C95" s="18" t="s">
+        <v>459</v>
+      </c>
+      <c r="D95" s="18" t="s">
+        <v>460</v>
+      </c>
+      <c r="E95" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F95" s="18" t="s">
         <v>461</v>
       </c>
-      <c r="B95" s="18" t="s">
+      <c r="G95" s="18" t="s">
         <v>462</v>
       </c>
-      <c r="C95" s="18" t="s">
-        <v>463</v>
-      </c>
-      <c r="D95" s="18" t="s">
-        <v>464</v>
-      </c>
-      <c r="E95" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F95" s="18" t="s">
-        <v>465</v>
-      </c>
-      <c r="G95" s="18" t="s">
-        <v>466</v>
-      </c>
       <c r="H95" s="20">
-        <v>1548</v>
+        <v>1091</v>
       </c>
       <c r="I95" s="18" t="s">
         <v>28</v>
@@ -4877,28 +4862,28 @@
     </row>
     <row r="96" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A96" s="21" t="s">
+        <v>463</v>
+      </c>
+      <c r="B96" s="22" t="s">
+        <v>458</v>
+      </c>
+      <c r="C96" s="22" t="s">
+        <v>464</v>
+      </c>
+      <c r="D96" s="22" t="s">
+        <v>465</v>
+      </c>
+      <c r="E96" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F96" s="22" t="s">
+        <v>466</v>
+      </c>
+      <c r="G96" s="22" t="s">
         <v>467</v>
       </c>
-      <c r="B96" s="22" t="s">
-        <v>462</v>
-      </c>
-      <c r="C96" s="22" t="s">
-        <v>468</v>
-      </c>
-      <c r="D96" s="22" t="s">
-        <v>469</v>
-      </c>
-      <c r="E96" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F96" s="22" t="s">
-        <v>470</v>
-      </c>
-      <c r="G96" s="22" t="s">
-        <v>471</v>
-      </c>
       <c r="H96" s="23">
-        <v>868</v>
+        <v>1010</v>
       </c>
       <c r="I96" s="22" t="s">
         <v>28</v>
@@ -4906,28 +4891,28 @@
     </row>
     <row r="97" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A97" s="17" t="s">
+        <v>468</v>
+      </c>
+      <c r="B97" s="18" t="s">
+        <v>458</v>
+      </c>
+      <c r="C97" s="18" t="s">
+        <v>469</v>
+      </c>
+      <c r="D97" s="18" t="s">
+        <v>470</v>
+      </c>
+      <c r="E97" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F97" s="18" t="s">
+        <v>471</v>
+      </c>
+      <c r="G97" s="18" t="s">
         <v>472</v>
       </c>
-      <c r="B97" s="18" t="s">
-        <v>462</v>
-      </c>
-      <c r="C97" s="18" t="s">
-        <v>473</v>
-      </c>
-      <c r="D97" s="18" t="s">
-        <v>474</v>
-      </c>
-      <c r="E97" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F97" s="18" t="s">
-        <v>475</v>
-      </c>
-      <c r="G97" s="18" t="s">
-        <v>476</v>
-      </c>
       <c r="H97" s="20">
-        <v>479</v>
+        <v>1109</v>
       </c>
       <c r="I97" s="18" t="s">
         <v>28</v>
@@ -4935,28 +4920,28 @@
     </row>
     <row r="98" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A98" s="21" t="s">
+        <v>473</v>
+      </c>
+      <c r="B98" s="22" t="s">
+        <v>458</v>
+      </c>
+      <c r="C98" s="22" t="s">
+        <v>474</v>
+      </c>
+      <c r="D98" s="22" t="s">
+        <v>475</v>
+      </c>
+      <c r="E98" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F98" s="22" t="s">
+        <v>476</v>
+      </c>
+      <c r="G98" s="22" t="s">
         <v>477</v>
       </c>
-      <c r="B98" s="22" t="s">
-        <v>462</v>
-      </c>
-      <c r="C98" s="22" t="s">
-        <v>478</v>
-      </c>
-      <c r="D98" s="22" t="s">
-        <v>479</v>
-      </c>
-      <c r="E98" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F98" s="22" t="s">
-        <v>480</v>
-      </c>
-      <c r="G98" s="22" t="s">
-        <v>481</v>
-      </c>
       <c r="H98" s="23">
-        <v>1176</v>
+        <v>614</v>
       </c>
       <c r="I98" s="22" t="s">
         <v>28</v>
@@ -4964,28 +4949,28 @@
     </row>
     <row r="99" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A99" s="17" t="s">
+        <v>478</v>
+      </c>
+      <c r="B99" s="18" t="s">
+        <v>458</v>
+      </c>
+      <c r="C99" s="18" t="s">
+        <v>479</v>
+      </c>
+      <c r="D99" s="18" t="s">
+        <v>480</v>
+      </c>
+      <c r="E99" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F99" s="18" t="s">
+        <v>481</v>
+      </c>
+      <c r="G99" s="18" t="s">
         <v>482</v>
       </c>
-      <c r="B99" s="18" t="s">
-        <v>462</v>
-      </c>
-      <c r="C99" s="18" t="s">
-        <v>483</v>
-      </c>
-      <c r="D99" s="18" t="s">
-        <v>484</v>
-      </c>
-      <c r="E99" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F99" s="18" t="s">
-        <v>485</v>
-      </c>
-      <c r="G99" s="18" t="s">
-        <v>486</v>
-      </c>
       <c r="H99" s="20">
-        <v>1032</v>
+        <v>927</v>
       </c>
       <c r="I99" s="18" t="s">
         <v>28</v>
@@ -4993,28 +4978,28 @@
     </row>
     <row r="100" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100" s="21" t="s">
+        <v>483</v>
+      </c>
+      <c r="B100" s="22" t="s">
+        <v>458</v>
+      </c>
+      <c r="C100" s="22" t="s">
+        <v>484</v>
+      </c>
+      <c r="D100" s="22" t="s">
+        <v>485</v>
+      </c>
+      <c r="E100" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F100" s="22" t="s">
+        <v>486</v>
+      </c>
+      <c r="G100" s="22" t="s">
         <v>487</v>
       </c>
-      <c r="B100" s="22" t="s">
-        <v>462</v>
-      </c>
-      <c r="C100" s="22" t="s">
-        <v>488</v>
-      </c>
-      <c r="D100" s="22" t="s">
-        <v>489</v>
-      </c>
-      <c r="E100" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F100" s="22" t="s">
-        <v>490</v>
-      </c>
-      <c r="G100" s="22" t="s">
-        <v>491</v>
-      </c>
       <c r="H100" s="23">
-        <v>748</v>
+        <v>1236</v>
       </c>
       <c r="I100" s="22" t="s">
         <v>28</v>
@@ -5022,28 +5007,28 @@
     </row>
     <row r="101" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101" s="17" t="s">
+        <v>488</v>
+      </c>
+      <c r="B101" s="18" t="s">
+        <v>458</v>
+      </c>
+      <c r="C101" s="18" t="s">
+        <v>489</v>
+      </c>
+      <c r="D101" s="18" t="s">
+        <v>490</v>
+      </c>
+      <c r="E101" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F101" s="18" t="s">
+        <v>491</v>
+      </c>
+      <c r="G101" s="18" t="s">
         <v>492</v>
       </c>
-      <c r="B101" s="18" t="s">
-        <v>462</v>
-      </c>
-      <c r="C101" s="18" t="s">
-        <v>493</v>
-      </c>
-      <c r="D101" s="18" t="s">
-        <v>494</v>
-      </c>
-      <c r="E101" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F101" s="18" t="s">
-        <v>495</v>
-      </c>
-      <c r="G101" s="18" t="s">
-        <v>496</v>
-      </c>
       <c r="H101" s="20">
-        <v>1588</v>
+        <v>1282</v>
       </c>
       <c r="I101" s="18" t="s">
         <v>28</v>
@@ -5051,28 +5036,28 @@
     </row>
     <row r="102" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A102" s="21" t="s">
+        <v>493</v>
+      </c>
+      <c r="B102" s="22" t="s">
+        <v>458</v>
+      </c>
+      <c r="C102" s="22" t="s">
+        <v>494</v>
+      </c>
+      <c r="D102" s="22" t="s">
+        <v>495</v>
+      </c>
+      <c r="E102" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F102" s="22" t="s">
+        <v>496</v>
+      </c>
+      <c r="G102" s="22" t="s">
         <v>497</v>
       </c>
-      <c r="B102" s="22" t="s">
-        <v>462</v>
-      </c>
-      <c r="C102" s="22" t="s">
-        <v>498</v>
-      </c>
-      <c r="D102" s="22" t="s">
-        <v>499</v>
-      </c>
-      <c r="E102" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F102" s="22" t="s">
-        <v>500</v>
-      </c>
-      <c r="G102" s="22" t="s">
-        <v>501</v>
-      </c>
       <c r="H102" s="23">
-        <v>1357</v>
+        <v>1055</v>
       </c>
       <c r="I102" s="22" t="s">
         <v>28</v>
@@ -5080,28 +5065,28 @@
     </row>
     <row r="103" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A103" s="17" t="s">
+        <v>498</v>
+      </c>
+      <c r="B103" s="18" t="s">
+        <v>499</v>
+      </c>
+      <c r="C103" s="18" t="s">
+        <v>500</v>
+      </c>
+      <c r="D103" s="18" t="s">
+        <v>501</v>
+      </c>
+      <c r="E103" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F103" s="18" t="s">
         <v>502</v>
       </c>
-      <c r="B103" s="18" t="s">
+      <c r="G103" s="18" t="s">
         <v>503</v>
       </c>
-      <c r="C103" s="18" t="s">
-        <v>504</v>
-      </c>
-      <c r="D103" s="18" t="s">
-        <v>505</v>
-      </c>
-      <c r="E103" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F103" s="18" t="s">
-        <v>506</v>
-      </c>
-      <c r="G103" s="18" t="s">
-        <v>507</v>
-      </c>
       <c r="H103" s="20">
-        <v>372</v>
+        <v>737</v>
       </c>
       <c r="I103" s="18" t="s">
         <v>28</v>
@@ -5109,28 +5094,28 @@
     </row>
     <row r="104" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A104" s="21" t="s">
+        <v>504</v>
+      </c>
+      <c r="B104" s="22" t="s">
+        <v>499</v>
+      </c>
+      <c r="C104" s="22" t="s">
+        <v>505</v>
+      </c>
+      <c r="D104" s="22" t="s">
+        <v>506</v>
+      </c>
+      <c r="E104" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F104" s="22" t="s">
+        <v>507</v>
+      </c>
+      <c r="G104" s="22" t="s">
         <v>508</v>
       </c>
-      <c r="B104" s="22" t="s">
-        <v>503</v>
-      </c>
-      <c r="C104" s="22" t="s">
-        <v>509</v>
-      </c>
-      <c r="D104" s="22" t="s">
-        <v>510</v>
-      </c>
-      <c r="E104" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F104" s="22" t="s">
-        <v>511</v>
-      </c>
-      <c r="G104" s="22" t="s">
-        <v>512</v>
-      </c>
       <c r="H104" s="23">
-        <v>1496</v>
+        <v>718</v>
       </c>
       <c r="I104" s="22" t="s">
         <v>28</v>
@@ -5138,28 +5123,28 @@
     </row>
     <row r="105" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A105" s="17" t="s">
-        <v>513</v>
+        <v>509</v>
       </c>
       <c r="B105" s="18" t="s">
-        <v>503</v>
+        <v>499</v>
       </c>
       <c r="C105" s="18" t="s">
+        <v>510</v>
+      </c>
+      <c r="D105" s="18" t="s">
+        <v>511</v>
+      </c>
+      <c r="E105" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F105" s="18" t="s">
+        <v>292</v>
+      </c>
+      <c r="G105" s="18" t="s">
+        <v>512</v>
+      </c>
+      <c r="H105" s="20">
         <v>514</v>
-      </c>
-      <c r="D105" s="18" t="s">
-        <v>515</v>
-      </c>
-      <c r="E105" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F105" s="18" t="s">
-        <v>516</v>
-      </c>
-      <c r="G105" s="18" t="s">
-        <v>517</v>
-      </c>
-      <c r="H105" s="20">
-        <v>1291</v>
       </c>
       <c r="I105" s="18" t="s">
         <v>28</v>
@@ -5167,28 +5152,28 @@
     </row>
     <row r="106" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A106" s="21" t="s">
-        <v>518</v>
+        <v>513</v>
       </c>
       <c r="B106" s="22" t="s">
-        <v>503</v>
+        <v>499</v>
       </c>
       <c r="C106" s="22" t="s">
-        <v>519</v>
+        <v>514</v>
       </c>
       <c r="D106" s="22" t="s">
-        <v>520</v>
+        <v>515</v>
       </c>
       <c r="E106" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F106" s="22" t="s">
-        <v>521</v>
+        <v>516</v>
       </c>
       <c r="G106" s="22" t="s">
-        <v>522</v>
+        <v>517</v>
       </c>
       <c r="H106" s="23">
-        <v>1658</v>
+        <v>566</v>
       </c>
       <c r="I106" s="22" t="s">
         <v>28</v>
@@ -5196,28 +5181,28 @@
     </row>
     <row r="107" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A107" s="17" t="s">
-        <v>523</v>
+        <v>518</v>
       </c>
       <c r="B107" s="18" t="s">
-        <v>503</v>
+        <v>499</v>
       </c>
       <c r="C107" s="18" t="s">
-        <v>524</v>
+        <v>519</v>
       </c>
       <c r="D107" s="18" t="s">
-        <v>525</v>
+        <v>520</v>
       </c>
       <c r="E107" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F107" s="18" t="s">
-        <v>526</v>
+        <v>521</v>
       </c>
       <c r="G107" s="18" t="s">
-        <v>527</v>
+        <v>522</v>
       </c>
       <c r="H107" s="20">
-        <v>1404</v>
+        <v>1595</v>
       </c>
       <c r="I107" s="18" t="s">
         <v>28</v>
@@ -5225,28 +5210,28 @@
     </row>
     <row r="108" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A108" s="21" t="s">
-        <v>528</v>
+        <v>523</v>
       </c>
       <c r="B108" s="22" t="s">
-        <v>503</v>
+        <v>499</v>
       </c>
       <c r="C108" s="22" t="s">
-        <v>529</v>
+        <v>524</v>
       </c>
       <c r="D108" s="22" t="s">
-        <v>530</v>
+        <v>525</v>
       </c>
       <c r="E108" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F108" s="22" t="s">
-        <v>531</v>
+        <v>526</v>
       </c>
       <c r="G108" s="22" t="s">
-        <v>532</v>
+        <v>527</v>
       </c>
       <c r="H108" s="23">
-        <v>1353</v>
+        <v>1249</v>
       </c>
       <c r="I108" s="22" t="s">
         <v>28</v>

</xml_diff>